<commit_message>
Fase 2 sincronizada: EP-21 y 12 historias nuevas, Sprint 5 cerrado, avance web del Sprint 6, informes de prueba S5/S6, ceremonias del S5
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Fase 2/Evidencias Proyecto/SIGMA_Product_Backlog_por_Sprint.xlsx
+++ b/Fase 2/Evidencias Proyecto/SIGMA_Product_Backlog_por_Sprint.xlsx
@@ -1224,19 +1224,19 @@
     </row>
     <row r="21" ht="30" customHeight="1" s="26">
       <c r="B21" s="7">
-        <f>COUNTA(Épicas!A6:A25)</f>
+        <f>COUNTA(Épicas!A6:A26)</f>
         <v/>
       </c>
       <c r="C21" s="7">
-        <f>COUNTA('Backlog completo'!A6:A137)</f>
+        <f>COUNTA('Backlog completo'!A6:A155)</f>
         <v/>
       </c>
       <c r="D21" s="7">
-        <f>SUM('Backlog completo'!J6:J137)</f>
+        <f>SUM('Backlog completo'!J6:J155)</f>
         <v/>
       </c>
       <c r="E21" s="7">
-        <f>COUNTA('Criterios de aceptación'!A6:A391)</f>
+        <f>COUNTA('Criterios de aceptación'!A6:A442)</f>
         <v/>
       </c>
       <c r="F21" s="7">
@@ -1319,11 +1319,11 @@
         </is>
       </c>
       <c r="F25" s="9">
-        <f>COUNTIF('Backlog completo'!$L$6:$L$143,$B25)</f>
+        <f>COUNTIF('Backlog completo'!$L$6:$L$155,$B25)</f>
         <v/>
       </c>
       <c r="G25" s="9">
-        <f>SUMIF('Backlog completo'!$L$6:$L$143,$B25,'Backlog completo'!$J$6:$J$143)</f>
+        <f>SUMIF('Backlog completo'!$L$6:$L$155,$B25,'Backlog completo'!$J$6:$J$155)</f>
         <v/>
       </c>
       <c r="H25" s="11">
@@ -1357,11 +1357,11 @@
         </is>
       </c>
       <c r="F26" s="12">
-        <f>COUNTIF('Backlog completo'!$L$6:$L$143,$B26)</f>
+        <f>COUNTIF('Backlog completo'!$L$6:$L$155,$B26)</f>
         <v/>
       </c>
       <c r="G26" s="12">
-        <f>SUMIF('Backlog completo'!$L$6:$L$143,$B26,'Backlog completo'!$J$6:$J$143)</f>
+        <f>SUMIF('Backlog completo'!$L$6:$L$155,$B26,'Backlog completo'!$J$6:$J$155)</f>
         <v/>
       </c>
       <c r="H26" s="14">
@@ -1395,11 +1395,11 @@
         </is>
       </c>
       <c r="F27" s="9">
-        <f>COUNTIF('Backlog completo'!$L$6:$L$143,$B27)</f>
+        <f>COUNTIF('Backlog completo'!$L$6:$L$155,$B27)</f>
         <v/>
       </c>
       <c r="G27" s="9">
-        <f>SUMIF('Backlog completo'!$L$6:$L$143,$B27,'Backlog completo'!$J$6:$J$143)</f>
+        <f>SUMIF('Backlog completo'!$L$6:$L$155,$B27,'Backlog completo'!$J$6:$J$155)</f>
         <v/>
       </c>
       <c r="H27" s="11">
@@ -1433,11 +1433,11 @@
         </is>
       </c>
       <c r="F28" s="12">
-        <f>COUNTIF('Backlog completo'!$L$6:$L$143,$B28)</f>
+        <f>COUNTIF('Backlog completo'!$L$6:$L$155,$B28)</f>
         <v/>
       </c>
       <c r="G28" s="12">
-        <f>SUMIF('Backlog completo'!$L$6:$L$143,$B28,'Backlog completo'!$J$6:$J$143)</f>
+        <f>SUMIF('Backlog completo'!$L$6:$L$155,$B28,'Backlog completo'!$J$6:$J$155)</f>
         <v/>
       </c>
       <c r="H28" s="14">
@@ -1471,11 +1471,11 @@
         </is>
       </c>
       <c r="F29" s="9">
-        <f>COUNTIF('Backlog completo'!$L$6:$L$143,$B29)</f>
+        <f>COUNTIF('Backlog completo'!$L$6:$L$155,$B29)</f>
         <v/>
       </c>
       <c r="G29" s="9">
-        <f>SUMIF('Backlog completo'!$L$6:$L$143,$B29,'Backlog completo'!$J$6:$J$143)</f>
+        <f>SUMIF('Backlog completo'!$L$6:$L$155,$B29,'Backlog completo'!$J$6:$J$155)</f>
         <v/>
       </c>
       <c r="H29" s="11">
@@ -1509,11 +1509,11 @@
         </is>
       </c>
       <c r="F30" s="12">
-        <f>COUNTIF('Backlog completo'!$L$6:$L$143,$B30)</f>
+        <f>COUNTIF('Backlog completo'!$L$6:$L$155,$B30)</f>
         <v/>
       </c>
       <c r="G30" s="12">
-        <f>SUMIF('Backlog completo'!$L$6:$L$143,$B30,'Backlog completo'!$J$6:$J$143)</f>
+        <f>SUMIF('Backlog completo'!$L$6:$L$155,$B30,'Backlog completo'!$J$6:$J$155)</f>
         <v/>
       </c>
       <c r="H30" s="14">
@@ -1597,11 +1597,11 @@
         </is>
       </c>
       <c r="D35" s="9">
-        <f>COUNTIF('Backlog completo'!$K$6:$K$143,$B35)</f>
+        <f>COUNTIF('Backlog completo'!$K$6:$K$155,$B35)</f>
         <v/>
       </c>
       <c r="E35" s="9">
-        <f>SUMIF('Backlog completo'!$K$6:$K$143,$B35,'Backlog completo'!$J$6:$J$143)</f>
+        <f>SUMIF('Backlog completo'!$K$6:$K$155,$B35,'Backlog completo'!$J$6:$J$155)</f>
         <v/>
       </c>
       <c r="F35" s="11">
@@ -1621,11 +1621,11 @@
         </is>
       </c>
       <c r="D36" s="12">
-        <f>COUNTIF('Backlog completo'!$K$6:$K$143,$B36)</f>
+        <f>COUNTIF('Backlog completo'!$K$6:$K$155,$B36)</f>
         <v/>
       </c>
       <c r="E36" s="12">
-        <f>SUMIF('Backlog completo'!$K$6:$K$143,$B36,'Backlog completo'!$J$6:$J$143)</f>
+        <f>SUMIF('Backlog completo'!$K$6:$K$155,$B36,'Backlog completo'!$J$6:$J$155)</f>
         <v/>
       </c>
       <c r="F36" s="14">
@@ -1645,11 +1645,11 @@
         </is>
       </c>
       <c r="D37" s="9">
-        <f>COUNTIF('Backlog completo'!$K$6:$K$143,$B37)</f>
+        <f>COUNTIF('Backlog completo'!$K$6:$K$155,$B37)</f>
         <v/>
       </c>
       <c r="E37" s="9">
-        <f>SUMIF('Backlog completo'!$K$6:$K$143,$B37,'Backlog completo'!$J$6:$J$143)</f>
+        <f>SUMIF('Backlog completo'!$K$6:$K$155,$B37,'Backlog completo'!$J$6:$J$155)</f>
         <v/>
       </c>
       <c r="F37" s="11">
@@ -1696,7 +1696,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:O143"/>
+  <dimension ref="A1:O155"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" style="26" min="1" max="1"/>
@@ -11315,6 +11315,828 @@
         <v>4</v>
       </c>
       <c r="O143" s="9" t="n"/>
+    </row>
+    <row r="144">
+      <c r="A144" s="9" t="inlineStr">
+        <is>
+          <t>HU-210</t>
+        </is>
+      </c>
+      <c r="B144" s="9" t="inlineStr">
+        <is>
+          <t>EP-21</t>
+        </is>
+      </c>
+      <c r="C144" s="10" t="inlineStr">
+        <is>
+          <t>Operación comercial y de plataforma</t>
+        </is>
+      </c>
+      <c r="D144" s="10" t="inlineStr">
+        <is>
+          <t>Gestionar los leads en el pipeline comercial</t>
+        </is>
+      </c>
+      <c r="E144" s="10" t="inlineStr">
+        <is>
+          <t>ejecutivo comercial de SIGMA</t>
+        </is>
+      </c>
+      <c r="F144" s="10" t="inlineStr">
+        <is>
+          <t>registrar un lead con su país e identificador y llevarlo por etapas hasta concretarlo</t>
+        </is>
+      </c>
+      <c r="G144" s="10" t="inlineStr">
+        <is>
+          <t>no perder el seguimiento de ningún prospecto y saber cuánto hay en cada etapa</t>
+        </is>
+      </c>
+      <c r="H144" s="9" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="I144" s="9" t="n">
+        <v>90</v>
+      </c>
+      <c r="J144" s="9" t="n">
+        <v>8</v>
+      </c>
+      <c r="K144" s="9" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="L144" s="9" t="inlineStr">
+        <is>
+          <t>Sprint 5</t>
+        </is>
+      </c>
+      <c r="M144" s="10" t="inlineStr">
+        <is>
+          <t>HU-190</t>
+        </is>
+      </c>
+      <c r="N144" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="O144" s="9" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="9" t="inlineStr">
+        <is>
+          <t>HU-211</t>
+        </is>
+      </c>
+      <c r="B145" s="9" t="inlineStr">
+        <is>
+          <t>EP-21</t>
+        </is>
+      </c>
+      <c r="C145" s="10" t="inlineStr">
+        <is>
+          <t>Operación comercial y de plataforma</t>
+        </is>
+      </c>
+      <c r="D145" s="10" t="inlineStr">
+        <is>
+          <t>Enviar la propuesta y generar el contrato</t>
+        </is>
+      </c>
+      <c r="E145" s="10" t="inlineStr">
+        <is>
+          <t>ejecutivo comercial de SIGMA</t>
+        </is>
+      </c>
+      <c r="F145" s="10" t="inlineStr">
+        <is>
+          <t>armar una propuesta con plan estándar o personalizado y generar el contrato desde ella</t>
+        </is>
+      </c>
+      <c r="G145" s="10" t="inlineStr">
+        <is>
+          <t>que el cliente reciba una oferta clara y firmable, con sus versiones guardadas</t>
+        </is>
+      </c>
+      <c r="H145" s="9" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="I145" s="9" t="n">
+        <v>90</v>
+      </c>
+      <c r="J145" s="9" t="n">
+        <v>8</v>
+      </c>
+      <c r="K145" s="9" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="L145" s="9" t="inlineStr">
+        <is>
+          <t>Sprint 5</t>
+        </is>
+      </c>
+      <c r="M145" s="10" t="inlineStr">
+        <is>
+          <t>HU-210, HU-190</t>
+        </is>
+      </c>
+      <c r="N145" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="O145" s="9" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="9" t="inlineStr">
+        <is>
+          <t>HU-212</t>
+        </is>
+      </c>
+      <c r="B146" s="9" t="inlineStr">
+        <is>
+          <t>EP-21</t>
+        </is>
+      </c>
+      <c r="C146" s="10" t="inlineStr">
+        <is>
+          <t>Operación comercial y de plataforma</t>
+        </is>
+      </c>
+      <c r="D146" s="10" t="inlineStr">
+        <is>
+          <t>Firmar el contrato en línea</t>
+        </is>
+      </c>
+      <c r="E146" s="10" t="inlineStr">
+        <is>
+          <t>representante del cliente</t>
+        </is>
+      </c>
+      <c r="F146" s="10" t="inlineStr">
+        <is>
+          <t>leer el contrato y firmarlo desde el enlace que recibí por correo, sin crear una cuenta</t>
+        </is>
+      </c>
+      <c r="G146" s="10" t="inlineStr">
+        <is>
+          <t>dejar la contratación cerrada con respaldo legal sin trámites presenciales</t>
+        </is>
+      </c>
+      <c r="H146" s="9" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="I146" s="9" t="n">
+        <v>90</v>
+      </c>
+      <c r="J146" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="K146" s="9" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="L146" s="9" t="inlineStr">
+        <is>
+          <t>Sprint 5</t>
+        </is>
+      </c>
+      <c r="M146" s="10" t="inlineStr">
+        <is>
+          <t>HU-211</t>
+        </is>
+      </c>
+      <c r="N146" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="O146" s="9" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="9" t="inlineStr">
+        <is>
+          <t>HU-213</t>
+        </is>
+      </c>
+      <c r="B147" s="9" t="inlineStr">
+        <is>
+          <t>EP-21</t>
+        </is>
+      </c>
+      <c r="C147" s="10" t="inlineStr">
+        <is>
+          <t>Operación comercial y de plataforma</t>
+        </is>
+      </c>
+      <c r="D147" s="10" t="inlineStr">
+        <is>
+          <t>Cobrar la suscripción con Webpay o transferencia</t>
+        </is>
+      </c>
+      <c r="E147" s="10" t="inlineStr">
+        <is>
+          <t>administrador de SIGMA</t>
+        </is>
+      </c>
+      <c r="F147" s="10" t="inlineStr">
+        <is>
+          <t>emitir cada período de cobro y registrar su pago por Webpay o por transferencia verificada</t>
+        </is>
+      </c>
+      <c r="G147" s="10" t="inlineStr">
+        <is>
+          <t>saber qué cliente está al día y no perder ningún cobro</t>
+        </is>
+      </c>
+      <c r="H147" s="9" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="I147" s="9" t="n">
+        <v>90</v>
+      </c>
+      <c r="J147" s="9" t="n">
+        <v>8</v>
+      </c>
+      <c r="K147" s="9" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="L147" s="9" t="inlineStr">
+        <is>
+          <t>Sprint 5</t>
+        </is>
+      </c>
+      <c r="M147" s="10" t="inlineStr">
+        <is>
+          <t>HU-191, HU-212</t>
+        </is>
+      </c>
+      <c r="N147" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="O147" s="9" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="9" t="inlineStr">
+        <is>
+          <t>HU-214</t>
+        </is>
+      </c>
+      <c r="B148" s="9" t="inlineStr">
+        <is>
+          <t>EP-21</t>
+        </is>
+      </c>
+      <c r="C148" s="10" t="inlineStr">
+        <is>
+          <t>Operación comercial y de plataforma</t>
+        </is>
+      </c>
+      <c r="D148" s="10" t="inlineStr">
+        <is>
+          <t>Atender clientes de otros países</t>
+        </is>
+      </c>
+      <c r="E148" s="10" t="inlineStr">
+        <is>
+          <t>administrador de SIGMA</t>
+        </is>
+      </c>
+      <c r="F148" s="10" t="inlineStr">
+        <is>
+          <t>registrar empresas de Chile, Argentina, Colombia, Ecuador, México y Perú con su identificador, zona horaria y moneda</t>
+        </is>
+      </c>
+      <c r="G148" s="10" t="inlineStr">
+        <is>
+          <t>vender SIGMA fuera de Chile sin cambiar el sistema</t>
+        </is>
+      </c>
+      <c r="H148" s="9" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="I148" s="9" t="n">
+        <v>75</v>
+      </c>
+      <c r="J148" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="K148" s="9" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="L148" s="9" t="inlineStr">
+        <is>
+          <t>Sprint 5</t>
+        </is>
+      </c>
+      <c r="M148" s="10" t="inlineStr">
+        <is>
+          <t>HU-210</t>
+        </is>
+      </c>
+      <c r="N148" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="O148" s="9" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="9" t="inlineStr">
+        <is>
+          <t>HU-215</t>
+        </is>
+      </c>
+      <c r="B149" s="9" t="inlineStr">
+        <is>
+          <t>EP-21</t>
+        </is>
+      </c>
+      <c r="C149" s="10" t="inlineStr">
+        <is>
+          <t>Operación comercial y de plataforma</t>
+        </is>
+      </c>
+      <c r="D149" s="10" t="inlineStr">
+        <is>
+          <t>Ejecutar los procesos automáticos de SIGMA</t>
+        </is>
+      </c>
+      <c r="E149" s="10" t="inlineStr">
+        <is>
+          <t>administrador de SIGMA</t>
+        </is>
+      </c>
+      <c r="F149" s="10" t="inlineStr">
+        <is>
+          <t>que ocurrencias, órdenes automáticas, cobros, alertas, UF y vencimiento de demos corran solos cada cierto tiempo</t>
+        </is>
+      </c>
+      <c r="G149" s="10" t="inlineStr">
+        <is>
+          <t>no depender de que alguien abra la web ni de un servidor con agendador</t>
+        </is>
+      </c>
+      <c r="H149" s="9" t="inlineStr">
+        <is>
+          <t>Web (infraestructura)</t>
+        </is>
+      </c>
+      <c r="I149" s="9" t="n">
+        <v>90</v>
+      </c>
+      <c r="J149" s="9" t="n">
+        <v>8</v>
+      </c>
+      <c r="K149" s="9" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="L149" s="9" t="inlineStr">
+        <is>
+          <t>Sprint 5</t>
+        </is>
+      </c>
+      <c r="M149" s="10" t="inlineStr">
+        <is>
+          <t>HU-094, HU-111</t>
+        </is>
+      </c>
+      <c r="N149" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="O149" s="9" t="n"/>
+    </row>
+    <row r="150">
+      <c r="A150" s="9" t="inlineStr">
+        <is>
+          <t>HU-216</t>
+        </is>
+      </c>
+      <c r="B150" s="9" t="inlineStr">
+        <is>
+          <t>EP-21</t>
+        </is>
+      </c>
+      <c r="C150" s="10" t="inlineStr">
+        <is>
+          <t>Operación comercial y de plataforma</t>
+        </is>
+      </c>
+      <c r="D150" s="10" t="inlineStr">
+        <is>
+          <t>Enviar los correos con reintentos y copia de monitoreo</t>
+        </is>
+      </c>
+      <c r="E150" s="10" t="inlineStr">
+        <is>
+          <t>administrador de SIGMA</t>
+        </is>
+      </c>
+      <c r="F150" s="10" t="inlineStr">
+        <is>
+          <t>que todo correo del sistema pase por una cola con reintentos y que yo reciba copia oculta</t>
+        </is>
+      </c>
+      <c r="G150" s="10" t="inlineStr">
+        <is>
+          <t>que un fallo del servidor de correo no pierda mensajes y poder vigilar lo que se envía</t>
+        </is>
+      </c>
+      <c r="H150" s="9" t="inlineStr">
+        <is>
+          <t>Web (infraestructura)</t>
+        </is>
+      </c>
+      <c r="I150" s="9" t="n">
+        <v>80</v>
+      </c>
+      <c r="J150" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="K150" s="9" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="L150" s="9" t="inlineStr">
+        <is>
+          <t>Sprint 5</t>
+        </is>
+      </c>
+      <c r="M150" s="10" t="inlineStr">
+        <is>
+          <t>HU-215</t>
+        </is>
+      </c>
+      <c r="N150" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="O150" s="9" t="n"/>
+    </row>
+    <row r="151">
+      <c r="A151" s="9" t="inlineStr">
+        <is>
+          <t>HU-217</t>
+        </is>
+      </c>
+      <c r="B151" s="9" t="inlineStr">
+        <is>
+          <t>EP-21</t>
+        </is>
+      </c>
+      <c r="C151" s="10" t="inlineStr">
+        <is>
+          <t>Operación comercial y de plataforma</t>
+        </is>
+      </c>
+      <c r="D151" s="10" t="inlineStr">
+        <is>
+          <t>Reportar un problema y consultar la ayuda de la pantalla</t>
+        </is>
+      </c>
+      <c r="E151" s="10" t="inlineStr">
+        <is>
+          <t>usuario de SIGMA</t>
+        </is>
+      </c>
+      <c r="F151" s="10" t="inlineStr">
+        <is>
+          <t>reportar un problema desde cualquier pantalla y leer la ayuda contextual de esa pantalla</t>
+        </is>
+      </c>
+      <c r="G151" s="10" t="inlineStr">
+        <is>
+          <t>resolver mis dudas sin llamar y que soporte reciba el contexto</t>
+        </is>
+      </c>
+      <c r="H151" s="9" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="I151" s="9" t="n">
+        <v>85</v>
+      </c>
+      <c r="J151" s="9" t="n">
+        <v>8</v>
+      </c>
+      <c r="K151" s="9" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="L151" s="9" t="inlineStr">
+        <is>
+          <t>Sprint 5</t>
+        </is>
+      </c>
+      <c r="M151" s="10" t="inlineStr">
+        <is>
+          <t>HU-006</t>
+        </is>
+      </c>
+      <c r="N151" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="O151" s="9" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="9" t="inlineStr">
+        <is>
+          <t>HU-218</t>
+        </is>
+      </c>
+      <c r="B152" s="9" t="inlineStr">
+        <is>
+          <t>EP-21</t>
+        </is>
+      </c>
+      <c r="C152" s="10" t="inlineStr">
+        <is>
+          <t>Operación comercial y de plataforma</t>
+        </is>
+      </c>
+      <c r="D152" s="10" t="inlineStr">
+        <is>
+          <t>Atender los tickets de soporte con plazos y encuesta</t>
+        </is>
+      </c>
+      <c r="E152" s="10" t="inlineStr">
+        <is>
+          <t>administrador de SIGMA</t>
+        </is>
+      </c>
+      <c r="F152" s="10" t="inlineStr">
+        <is>
+          <t>gestionar los tickets con prioridad, plazo de respuesta (SLA) y encuesta de satisfacción</t>
+        </is>
+      </c>
+      <c r="G152" s="10" t="inlineStr">
+        <is>
+          <t>cumplir lo prometido al cliente y medir la calidad del servicio</t>
+        </is>
+      </c>
+      <c r="H152" s="9" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="I152" s="9" t="n">
+        <v>80</v>
+      </c>
+      <c r="J152" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="K152" s="9" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="L152" s="9" t="inlineStr">
+        <is>
+          <t>Sprint 5</t>
+        </is>
+      </c>
+      <c r="M152" s="10" t="inlineStr">
+        <is>
+          <t>HU-217</t>
+        </is>
+      </c>
+      <c r="N152" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="O152" s="9" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" s="9" t="inlineStr">
+        <is>
+          <t>HU-219</t>
+        </is>
+      </c>
+      <c r="B153" s="9" t="inlineStr">
+        <is>
+          <t>EP-21</t>
+        </is>
+      </c>
+      <c r="C153" s="10" t="inlineStr">
+        <is>
+          <t>Operación comercial y de plataforma</t>
+        </is>
+      </c>
+      <c r="D153" s="10" t="inlineStr">
+        <is>
+          <t>Comunicar novedades con campañas segmentadas</t>
+        </is>
+      </c>
+      <c r="E153" s="10" t="inlineStr">
+        <is>
+          <t>administrador de SIGMA</t>
+        </is>
+      </c>
+      <c r="F153" s="10" t="inlineStr">
+        <is>
+          <t>publicar un aviso (banner, modal o tarjeta) a un grupo de usuarios definido por estado, perfil, cliente o planta</t>
+        </is>
+      </c>
+      <c r="G153" s="10" t="inlineStr">
+        <is>
+          <t>informar cambios y novedades solo a quienes les corresponden</t>
+        </is>
+      </c>
+      <c r="H153" s="9" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="I153" s="9" t="n">
+        <v>65</v>
+      </c>
+      <c r="J153" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="K153" s="9" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="L153" s="9" t="inlineStr">
+        <is>
+          <t>Sprint 5</t>
+        </is>
+      </c>
+      <c r="M153" s="10" t="inlineStr">
+        <is>
+          <t>HU-217</t>
+        </is>
+      </c>
+      <c r="N153" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="O153" s="9" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="9" t="inlineStr">
+        <is>
+          <t>HU-220</t>
+        </is>
+      </c>
+      <c r="B154" s="9" t="inlineStr">
+        <is>
+          <t>EP-06</t>
+        </is>
+      </c>
+      <c r="C154" s="10" t="inlineStr">
+        <is>
+          <t>Repuestos, bodegas e inventario</t>
+        </is>
+      </c>
+      <c r="D154" s="10" t="inlineStr">
+        <is>
+          <t>Recorrer y operar la bodega en 3D (SIGMA Twin)</t>
+        </is>
+      </c>
+      <c r="E154" s="10" t="inlineStr">
+        <is>
+          <t>bodeguero</t>
+        </is>
+      </c>
+      <c r="F154" s="10" t="inlineStr">
+        <is>
+          <t>ver mis bodegas como un gemelo digital, preparar un picking y contar desde el recorrido</t>
+        </is>
+      </c>
+      <c r="G154" s="10" t="inlineStr">
+        <is>
+          <t>ubicar cada repuesto sin buscar y mantener el inventario exacto</t>
+        </is>
+      </c>
+      <c r="H154" s="9" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="I154" s="9" t="n">
+        <v>85</v>
+      </c>
+      <c r="J154" s="9" t="n">
+        <v>8</v>
+      </c>
+      <c r="K154" s="9" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="L154" s="9" t="inlineStr">
+        <is>
+          <t>Sprint 5</t>
+        </is>
+      </c>
+      <c r="M154" s="10" t="inlineStr">
+        <is>
+          <t>HU-050, HU-059</t>
+        </is>
+      </c>
+      <c r="N154" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="O154" s="9" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="9" t="inlineStr">
+        <is>
+          <t>HU-221</t>
+        </is>
+      </c>
+      <c r="B155" s="9" t="inlineStr">
+        <is>
+          <t>EP-18</t>
+        </is>
+      </c>
+      <c r="C155" s="10" t="inlineStr">
+        <is>
+          <t>Indicadores de gestión</t>
+        </is>
+      </c>
+      <c r="D155" s="10" t="inlineStr">
+        <is>
+          <t>Ver mi inicio con accesos, alertas y SIGMA AI</t>
+        </is>
+      </c>
+      <c r="E155" s="10" t="inlineStr">
+        <is>
+          <t>usuario de SIGMA</t>
+        </is>
+      </c>
+      <c r="F155" s="10" t="inlineStr">
+        <is>
+          <t>un inicio con mis accesos directos, mis indicadores, mi turno y lo que requiere mi atención</t>
+        </is>
+      </c>
+      <c r="G155" s="10" t="inlineStr">
+        <is>
+          <t>empezar el día sabiendo qué hacer sin recorrer menús</t>
+        </is>
+      </c>
+      <c r="H155" s="9" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="I155" s="9" t="n">
+        <v>80</v>
+      </c>
+      <c r="J155" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="K155" s="9" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="L155" s="9" t="inlineStr">
+        <is>
+          <t>Sprint 5</t>
+        </is>
+      </c>
+      <c r="M155" s="10" t="inlineStr">
+        <is>
+          <t>HU-006</t>
+        </is>
+      </c>
+      <c r="N155" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="O155" s="9" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A5:O137"/>
@@ -11342,7 +12164,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G409"/>
+  <dimension ref="A1:G442"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" style="26" min="1" max="1"/>
@@ -26257,6 +27079,1194 @@
         <is>
           <t>Cuando la app consulta GET /alertas y /alertas/resumen
 Entonces recibe las mismas alertas y el mismo contador que la web</t>
+        </is>
+      </c>
+    </row>
+    <row r="410">
+      <c r="A410" s="12" t="inlineStr">
+        <is>
+          <t>HU-210</t>
+        </is>
+      </c>
+      <c r="B410" s="13" t="inlineStr">
+        <is>
+          <t>Gestionar los leads en el pipeline comercial</t>
+        </is>
+      </c>
+      <c r="C410" s="12" t="inlineStr">
+        <is>
+          <t>EP-21</t>
+        </is>
+      </c>
+      <c r="D410" s="12" t="inlineStr">
+        <is>
+          <t>Sprint 5</t>
+        </is>
+      </c>
+      <c r="E410" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="F410" s="13" t="inlineStr">
+        <is>
+          <t>Alta de un lead</t>
+        </is>
+      </c>
+      <c r="G410" s="13" t="inlineStr">
+        <is>
+          <t>Cuando registro un lead con empresa, contacto, correo, país e identificador
+Entonces queda en el pipeline en estado Contactado con su ejecutivo y su próxima acción</t>
+        </is>
+      </c>
+    </row>
+    <row r="411">
+      <c r="A411" s="12" t="inlineStr">
+        <is>
+          <t>HU-210</t>
+        </is>
+      </c>
+      <c r="B411" s="13" t="inlineStr">
+        <is>
+          <t>Gestionar los leads en el pipeline comercial</t>
+        </is>
+      </c>
+      <c r="C411" s="12" t="inlineStr">
+        <is>
+          <t>EP-21</t>
+        </is>
+      </c>
+      <c r="D411" s="12" t="inlineStr">
+        <is>
+          <t>Sprint 5</t>
+        </is>
+      </c>
+      <c r="E411" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="F411" s="13" t="inlineStr">
+        <is>
+          <t>Identificador según el país</t>
+        </is>
+      </c>
+      <c r="G411" s="13" t="inlineStr">
+        <is>
+          <t>Dado que elijo un país
+Entonces el identificador cambia de nombre (RUT, RUC, CUIT…) y se valida con las reglas de ese país</t>
+        </is>
+      </c>
+    </row>
+    <row r="412">
+      <c r="A412" s="12" t="inlineStr">
+        <is>
+          <t>HU-210</t>
+        </is>
+      </c>
+      <c r="B412" s="13" t="inlineStr">
+        <is>
+          <t>Gestionar los leads en el pipeline comercial</t>
+        </is>
+      </c>
+      <c r="C412" s="12" t="inlineStr">
+        <is>
+          <t>EP-21</t>
+        </is>
+      </c>
+      <c r="D412" s="12" t="inlineStr">
+        <is>
+          <t>Sprint 5</t>
+        </is>
+      </c>
+      <c r="E412" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="F412" s="13" t="inlineStr">
+        <is>
+          <t>Seguimiento por etapas</t>
+        </is>
+      </c>
+      <c r="G412" s="13" t="inlineStr">
+        <is>
+          <t>Cuando abro la ficha del lead
+Entonces veo sus etapas, la siguiente acción y las acciones disponibles según el estado</t>
+        </is>
+      </c>
+    </row>
+    <row r="413">
+      <c r="A413" s="12" t="inlineStr">
+        <is>
+          <t>HU-211</t>
+        </is>
+      </c>
+      <c r="B413" s="13" t="inlineStr">
+        <is>
+          <t>Enviar la propuesta y generar el contrato</t>
+        </is>
+      </c>
+      <c r="C413" s="12" t="inlineStr">
+        <is>
+          <t>EP-21</t>
+        </is>
+      </c>
+      <c r="D413" s="12" t="inlineStr">
+        <is>
+          <t>Sprint 5</t>
+        </is>
+      </c>
+      <c r="E413" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="F413" s="13" t="inlineStr">
+        <is>
+          <t>Propuesta con plan estándar</t>
+        </is>
+      </c>
+      <c r="G413" s="13" t="inlineStr">
+        <is>
+          <t>Cuando armo la propuesta eligiendo Básico, Medio o Full
+Entonces veo el precio en la moneda del cliente, la implementación, el descuento, la vigencia y el total</t>
+        </is>
+      </c>
+    </row>
+    <row r="414">
+      <c r="A414" s="12" t="inlineStr">
+        <is>
+          <t>HU-211</t>
+        </is>
+      </c>
+      <c r="B414" s="13" t="inlineStr">
+        <is>
+          <t>Enviar la propuesta y generar el contrato</t>
+        </is>
+      </c>
+      <c r="C414" s="12" t="inlineStr">
+        <is>
+          <t>EP-21</t>
+        </is>
+      </c>
+      <c r="D414" s="12" t="inlineStr">
+        <is>
+          <t>Sprint 5</t>
+        </is>
+      </c>
+      <c r="E414" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="F414" s="13" t="inlineStr">
+        <is>
+          <t>Plan personalizado</t>
+        </is>
+      </c>
+      <c r="G414" s="13" t="inlineStr">
+        <is>
+          <t>Cuando elijo un plan personalizado
+Entonces defino su nombre, los módulos incluidos y los límites</t>
+        </is>
+      </c>
+    </row>
+    <row r="415">
+      <c r="A415" s="12" t="inlineStr">
+        <is>
+          <t>HU-211</t>
+        </is>
+      </c>
+      <c r="B415" s="13" t="inlineStr">
+        <is>
+          <t>Enviar la propuesta y generar el contrato</t>
+        </is>
+      </c>
+      <c r="C415" s="12" t="inlineStr">
+        <is>
+          <t>EP-21</t>
+        </is>
+      </c>
+      <c r="D415" s="12" t="inlineStr">
+        <is>
+          <t>Sprint 5</t>
+        </is>
+      </c>
+      <c r="E415" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="F415" s="13" t="inlineStr">
+        <is>
+          <t>Contrato desde la propuesta</t>
+        </is>
+      </c>
+      <c r="G415" s="13" t="inlineStr">
+        <is>
+          <t>Cuando genero el contrato desde la propuesta enviada
+Entonces el contrato queda en versión 1 y la ficha ofrece el botón para enviarlo</t>
+        </is>
+      </c>
+    </row>
+    <row r="416">
+      <c r="A416" s="12" t="inlineStr">
+        <is>
+          <t>HU-212</t>
+        </is>
+      </c>
+      <c r="B416" s="13" t="inlineStr">
+        <is>
+          <t>Firmar el contrato en línea</t>
+        </is>
+      </c>
+      <c r="C416" s="12" t="inlineStr">
+        <is>
+          <t>EP-21</t>
+        </is>
+      </c>
+      <c r="D416" s="12" t="inlineStr">
+        <is>
+          <t>Sprint 5</t>
+        </is>
+      </c>
+      <c r="E416" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="F416" s="13" t="inlineStr">
+        <is>
+          <t>Lectura y firma</t>
+        </is>
+      </c>
+      <c r="G416" s="13" t="inlineStr">
+        <is>
+          <t>Cuando abro el enlace del correo
+Entonces veo el contrato y un resumen, y puedo firmar con mi nombre y mi cargo</t>
+        </is>
+      </c>
+    </row>
+    <row r="417">
+      <c r="A417" s="12" t="inlineStr">
+        <is>
+          <t>HU-212</t>
+        </is>
+      </c>
+      <c r="B417" s="13" t="inlineStr">
+        <is>
+          <t>Firmar el contrato en línea</t>
+        </is>
+      </c>
+      <c r="C417" s="12" t="inlineStr">
+        <is>
+          <t>EP-21</t>
+        </is>
+      </c>
+      <c r="D417" s="12" t="inlineStr">
+        <is>
+          <t>Sprint 5</t>
+        </is>
+      </c>
+      <c r="E417" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="F417" s="13" t="inlineStr">
+        <is>
+          <t>Enlace inválido</t>
+        </is>
+      </c>
+      <c r="G417" s="13" t="inlineStr">
+        <is>
+          <t>Dado un enlace alterado o vencido
+Entonces la página indica que el enlace no es válido y no muestra datos del contrato</t>
+        </is>
+      </c>
+    </row>
+    <row r="418">
+      <c r="A418" s="12" t="inlineStr">
+        <is>
+          <t>HU-212</t>
+        </is>
+      </c>
+      <c r="B418" s="13" t="inlineStr">
+        <is>
+          <t>Firmar el contrato en línea</t>
+        </is>
+      </c>
+      <c r="C418" s="12" t="inlineStr">
+        <is>
+          <t>EP-21</t>
+        </is>
+      </c>
+      <c r="D418" s="12" t="inlineStr">
+        <is>
+          <t>Sprint 5</t>
+        </is>
+      </c>
+      <c r="E418" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="F418" s="13" t="inlineStr">
+        <is>
+          <t>Respaldo de la firma</t>
+        </is>
+      </c>
+      <c r="G418" s="13" t="inlineStr">
+        <is>
+          <t>Cuando firmo
+Entonces queda registrada la fecha, la IP y la huella SHA-256 del documento firmado</t>
+        </is>
+      </c>
+    </row>
+    <row r="419">
+      <c r="A419" s="12" t="inlineStr">
+        <is>
+          <t>HU-213</t>
+        </is>
+      </c>
+      <c r="B419" s="13" t="inlineStr">
+        <is>
+          <t>Cobrar la suscripción con Webpay o transferencia</t>
+        </is>
+      </c>
+      <c r="C419" s="12" t="inlineStr">
+        <is>
+          <t>EP-21</t>
+        </is>
+      </c>
+      <c r="D419" s="12" t="inlineStr">
+        <is>
+          <t>Sprint 5</t>
+        </is>
+      </c>
+      <c r="E419" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="F419" s="13" t="inlineStr">
+        <is>
+          <t>Emisión del período</t>
+        </is>
+      </c>
+      <c r="G419" s="13" t="inlineStr">
+        <is>
+          <t>Cuando emito un período
+Entonces arranca donde terminó el anterior y congela el valor de la UF y el total en pesos</t>
+        </is>
+      </c>
+    </row>
+    <row r="420">
+      <c r="A420" s="12" t="inlineStr">
+        <is>
+          <t>HU-213</t>
+        </is>
+      </c>
+      <c r="B420" s="13" t="inlineStr">
+        <is>
+          <t>Cobrar la suscripción con Webpay o transferencia</t>
+        </is>
+      </c>
+      <c r="C420" s="12" t="inlineStr">
+        <is>
+          <t>EP-21</t>
+        </is>
+      </c>
+      <c r="D420" s="12" t="inlineStr">
+        <is>
+          <t>Sprint 5</t>
+        </is>
+      </c>
+      <c r="E420" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="F420" s="13" t="inlineStr">
+        <is>
+          <t>Pago con Webpay</t>
+        </is>
+      </c>
+      <c r="G420" s="13" t="inlineStr">
+        <is>
+          <t>Cuando el cliente paga con tarjeta
+Entonces el pago queda con su autorización, orden y período</t>
+        </is>
+      </c>
+    </row>
+    <row r="421">
+      <c r="A421" s="12" t="inlineStr">
+        <is>
+          <t>HU-213</t>
+        </is>
+      </c>
+      <c r="B421" s="13" t="inlineStr">
+        <is>
+          <t>Cobrar la suscripción con Webpay o transferencia</t>
+        </is>
+      </c>
+      <c r="C421" s="12" t="inlineStr">
+        <is>
+          <t>EP-21</t>
+        </is>
+      </c>
+      <c r="D421" s="12" t="inlineStr">
+        <is>
+          <t>Sprint 5</t>
+        </is>
+      </c>
+      <c r="E421" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="F421" s="13" t="inlineStr">
+        <is>
+          <t>Transferencia verificada</t>
+        </is>
+      </c>
+      <c r="G421" s="13" t="inlineStr">
+        <is>
+          <t>Cuando el cliente informa una transferencia
+Entonces aparece en «por verificar» y, al verificarla, el período queda pagado</t>
+        </is>
+      </c>
+    </row>
+    <row r="422">
+      <c r="A422" s="12" t="inlineStr">
+        <is>
+          <t>HU-213</t>
+        </is>
+      </c>
+      <c r="B422" s="13" t="inlineStr">
+        <is>
+          <t>Cobrar la suscripción con Webpay o transferencia</t>
+        </is>
+      </c>
+      <c r="C422" s="12" t="inlineStr">
+        <is>
+          <t>EP-21</t>
+        </is>
+      </c>
+      <c r="D422" s="12" t="inlineStr">
+        <is>
+          <t>Sprint 5</t>
+        </is>
+      </c>
+      <c r="E422" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="F422" s="13" t="inlineStr">
+        <is>
+          <t>El cliente ve su estado</t>
+        </is>
+      </c>
+      <c r="G422" s="13" t="inlineStr">
+        <is>
+          <t>Cuando el cliente abre Mi suscripción
+Entonces ve si está al día, su plan, su vigencia y el saldo pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="423">
+      <c r="A423" s="12" t="inlineStr">
+        <is>
+          <t>HU-214</t>
+        </is>
+      </c>
+      <c r="B423" s="13" t="inlineStr">
+        <is>
+          <t>Atender clientes de otros países</t>
+        </is>
+      </c>
+      <c r="C423" s="12" t="inlineStr">
+        <is>
+          <t>EP-21</t>
+        </is>
+      </c>
+      <c r="D423" s="12" t="inlineStr">
+        <is>
+          <t>Sprint 5</t>
+        </is>
+      </c>
+      <c r="E423" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="F423" s="13" t="inlineStr">
+        <is>
+          <t>Datos por país</t>
+        </is>
+      </c>
+      <c r="G423" s="13" t="inlineStr">
+        <is>
+          <t>Cuando abro una empresa
+Entonces veo su país, su identificador con el nombre local, su zona horaria y su moneda de cobro</t>
+        </is>
+      </c>
+    </row>
+    <row r="424">
+      <c r="A424" s="12" t="inlineStr">
+        <is>
+          <t>HU-214</t>
+        </is>
+      </c>
+      <c r="B424" s="13" t="inlineStr">
+        <is>
+          <t>Atender clientes de otros países</t>
+        </is>
+      </c>
+      <c r="C424" s="12" t="inlineStr">
+        <is>
+          <t>EP-21</t>
+        </is>
+      </c>
+      <c r="D424" s="12" t="inlineStr">
+        <is>
+          <t>Sprint 5</t>
+        </is>
+      </c>
+      <c r="E424" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="F424" s="13" t="inlineStr">
+        <is>
+          <t>Listado de empresas</t>
+        </is>
+      </c>
+      <c r="G424" s="13" t="inlineStr">
+        <is>
+          <t>Cuando consulto todas las empresas
+Entonces veo razón social, país, identificador y moneda de cobro</t>
+        </is>
+      </c>
+    </row>
+    <row r="425">
+      <c r="A425" s="12" t="inlineStr">
+        <is>
+          <t>HU-215</t>
+        </is>
+      </c>
+      <c r="B425" s="13" t="inlineStr">
+        <is>
+          <t>Ejecutar los procesos automáticos de SIGMA</t>
+        </is>
+      </c>
+      <c r="C425" s="12" t="inlineStr">
+        <is>
+          <t>EP-21</t>
+        </is>
+      </c>
+      <c r="D425" s="12" t="inlineStr">
+        <is>
+          <t>Sprint 5</t>
+        </is>
+      </c>
+      <c r="E425" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="F425" s="13" t="inlineStr">
+        <is>
+          <t>Ocurrencias y OT cada hora</t>
+        </is>
+      </c>
+      <c r="G425" s="13" t="inlineStr">
+        <is>
+          <t>Cuando pasa la hora configurada
+Entonces se generan las ocurrencias de los planes y las órdenes de trabajo automáticas que ya corresponde crear</t>
+        </is>
+      </c>
+    </row>
+    <row r="426">
+      <c r="A426" s="12" t="inlineStr">
+        <is>
+          <t>HU-215</t>
+        </is>
+      </c>
+      <c r="B426" s="13" t="inlineStr">
+        <is>
+          <t>Ejecutar los procesos automáticos de SIGMA</t>
+        </is>
+      </c>
+      <c r="C426" s="12" t="inlineStr">
+        <is>
+          <t>EP-21</t>
+        </is>
+      </c>
+      <c r="D426" s="12" t="inlineStr">
+        <is>
+          <t>Sprint 5</t>
+        </is>
+      </c>
+      <c r="E426" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="F426" s="13" t="inlineStr">
+        <is>
+          <t>Cobros automáticos</t>
+        </is>
+      </c>
+      <c r="G426" s="13" t="inlineStr">
+        <is>
+          <t>Cuando llega la fecha de un período
+Entonces se emite y se envían los recordatorios sin intervención</t>
+        </is>
+      </c>
+    </row>
+    <row r="427">
+      <c r="A427" s="12" t="inlineStr">
+        <is>
+          <t>HU-215</t>
+        </is>
+      </c>
+      <c r="B427" s="13" t="inlineStr">
+        <is>
+          <t>Ejecutar los procesos automáticos de SIGMA</t>
+        </is>
+      </c>
+      <c r="C427" s="12" t="inlineStr">
+        <is>
+          <t>EP-21</t>
+        </is>
+      </c>
+      <c r="D427" s="12" t="inlineStr">
+        <is>
+          <t>Sprint 5</t>
+        </is>
+      </c>
+      <c r="E427" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="F427" s="13" t="inlineStr">
+        <is>
+          <t>Registro de cada ejecución</t>
+        </is>
+      </c>
+      <c r="G427" s="13" t="inlineStr">
+        <is>
+          <t>Cuando corre un job
+Entonces queda su inicio, su fin, lo generado y el error si lo hubo</t>
+        </is>
+      </c>
+    </row>
+    <row r="428">
+      <c r="A428" s="12" t="inlineStr">
+        <is>
+          <t>HU-215</t>
+        </is>
+      </c>
+      <c r="B428" s="13" t="inlineStr">
+        <is>
+          <t>Ejecutar los procesos automáticos de SIGMA</t>
+        </is>
+      </c>
+      <c r="C428" s="12" t="inlineStr">
+        <is>
+          <t>EP-21</t>
+        </is>
+      </c>
+      <c r="D428" s="12" t="inlineStr">
+        <is>
+          <t>Sprint 5</t>
+        </is>
+      </c>
+      <c r="E428" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="F428" s="13" t="inlineStr">
+        <is>
+          <t>Despertar protegido</t>
+        </is>
+      </c>
+      <c r="G428" s="13" t="inlineStr">
+        <is>
+          <t>Cuando se llama a Jobs.aspx sin la clave
+Entonces no se ejecuta nada</t>
+        </is>
+      </c>
+    </row>
+    <row r="429">
+      <c r="A429" s="12" t="inlineStr">
+        <is>
+          <t>HU-216</t>
+        </is>
+      </c>
+      <c r="B429" s="13" t="inlineStr">
+        <is>
+          <t>Enviar los correos con reintentos y copia de monitoreo</t>
+        </is>
+      </c>
+      <c r="C429" s="12" t="inlineStr">
+        <is>
+          <t>EP-21</t>
+        </is>
+      </c>
+      <c r="D429" s="12" t="inlineStr">
+        <is>
+          <t>Sprint 5</t>
+        </is>
+      </c>
+      <c r="E429" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="F429" s="13" t="inlineStr">
+        <is>
+          <t>Cola con reintentos</t>
+        </is>
+      </c>
+      <c r="G429" s="13" t="inlineStr">
+        <is>
+          <t>Cuando el servidor de correo falla
+Entonces el mensaje queda en cola y se reintenta hasta cinco veces</t>
+        </is>
+      </c>
+    </row>
+    <row r="430">
+      <c r="A430" s="12" t="inlineStr">
+        <is>
+          <t>HU-216</t>
+        </is>
+      </c>
+      <c r="B430" s="13" t="inlineStr">
+        <is>
+          <t>Enviar los correos con reintentos y copia de monitoreo</t>
+        </is>
+      </c>
+      <c r="C430" s="12" t="inlineStr">
+        <is>
+          <t>EP-21</t>
+        </is>
+      </c>
+      <c r="D430" s="12" t="inlineStr">
+        <is>
+          <t>Sprint 5</t>
+        </is>
+      </c>
+      <c r="E430" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="F430" s="13" t="inlineStr">
+        <is>
+          <t>Copia de monitoreo</t>
+        </is>
+      </c>
+      <c r="G430" s="13" t="inlineStr">
+        <is>
+          <t>Dado que hay una dirección de monitoreo configurada
+Entonces recibe copia oculta y los destinatarios reales reciben el original</t>
+        </is>
+      </c>
+    </row>
+    <row r="431">
+      <c r="A431" s="12" t="inlineStr">
+        <is>
+          <t>HU-217</t>
+        </is>
+      </c>
+      <c r="B431" s="13" t="inlineStr">
+        <is>
+          <t>Reportar un problema y consultar la ayuda de la pantalla</t>
+        </is>
+      </c>
+      <c r="C431" s="12" t="inlineStr">
+        <is>
+          <t>EP-21</t>
+        </is>
+      </c>
+      <c r="D431" s="12" t="inlineStr">
+        <is>
+          <t>Sprint 5</t>
+        </is>
+      </c>
+      <c r="E431" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="F431" s="13" t="inlineStr">
+        <is>
+          <t>Reporte desde cualquier pantalla</t>
+        </is>
+      </c>
+      <c r="G431" s="13" t="inlineStr">
+        <is>
+          <t>Cuando reporto un problema
+Entonces el ticket queda con mi usuario, la pantalla, la categoría, la prioridad y mis adjuntos</t>
+        </is>
+      </c>
+    </row>
+    <row r="432">
+      <c r="A432" s="12" t="inlineStr">
+        <is>
+          <t>HU-217</t>
+        </is>
+      </c>
+      <c r="B432" s="13" t="inlineStr">
+        <is>
+          <t>Reportar un problema y consultar la ayuda de la pantalla</t>
+        </is>
+      </c>
+      <c r="C432" s="12" t="inlineStr">
+        <is>
+          <t>EP-21</t>
+        </is>
+      </c>
+      <c r="D432" s="12" t="inlineStr">
+        <is>
+          <t>Sprint 5</t>
+        </is>
+      </c>
+      <c r="E432" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="F432" s="13" t="inlineStr">
+        <is>
+          <t>Ayuda contextual</t>
+        </is>
+      </c>
+      <c r="G432" s="13" t="inlineStr">
+        <is>
+          <t>Cuando abro «? Ayuda» en una pantalla
+Entonces veo el contenido publicado de esa pantalla, sus pasos y recomendaciones</t>
+        </is>
+      </c>
+    </row>
+    <row r="433">
+      <c r="A433" s="12" t="inlineStr">
+        <is>
+          <t>HU-217</t>
+        </is>
+      </c>
+      <c r="B433" s="13" t="inlineStr">
+        <is>
+          <t>Reportar un problema y consultar la ayuda de la pantalla</t>
+        </is>
+      </c>
+      <c r="C433" s="12" t="inlineStr">
+        <is>
+          <t>EP-21</t>
+        </is>
+      </c>
+      <c r="D433" s="12" t="inlineStr">
+        <is>
+          <t>Sprint 5</t>
+        </is>
+      </c>
+      <c r="E433" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="F433" s="13" t="inlineStr">
+        <is>
+          <t>Cupo del plan</t>
+        </is>
+      </c>
+      <c r="G433" s="13" t="inlineStr">
+        <is>
+          <t>Dado que el plan limita los tickets por mes
+Entonces al superar el cupo el sistema lo indica</t>
+        </is>
+      </c>
+    </row>
+    <row r="434">
+      <c r="A434" s="12" t="inlineStr">
+        <is>
+          <t>HU-218</t>
+        </is>
+      </c>
+      <c r="B434" s="13" t="inlineStr">
+        <is>
+          <t>Atender los tickets de soporte con plazos y encuesta</t>
+        </is>
+      </c>
+      <c r="C434" s="12" t="inlineStr">
+        <is>
+          <t>EP-21</t>
+        </is>
+      </c>
+      <c r="D434" s="12" t="inlineStr">
+        <is>
+          <t>Sprint 5</t>
+        </is>
+      </c>
+      <c r="E434" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="F434" s="13" t="inlineStr">
+        <is>
+          <t>Gestión del ticket</t>
+        </is>
+      </c>
+      <c r="G434" s="13" t="inlineStr">
+        <is>
+          <t>Cuando atiendo un ticket
+Entonces cada cambio de estado queda en su historial con quién y cuándo</t>
+        </is>
+      </c>
+    </row>
+    <row r="435">
+      <c r="A435" s="12" t="inlineStr">
+        <is>
+          <t>HU-218</t>
+        </is>
+      </c>
+      <c r="B435" s="13" t="inlineStr">
+        <is>
+          <t>Atender los tickets de soporte con plazos y encuesta</t>
+        </is>
+      </c>
+      <c r="C435" s="12" t="inlineStr">
+        <is>
+          <t>EP-21</t>
+        </is>
+      </c>
+      <c r="D435" s="12" t="inlineStr">
+        <is>
+          <t>Sprint 5</t>
+        </is>
+      </c>
+      <c r="E435" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="F435" s="13" t="inlineStr">
+        <is>
+          <t>Plazo de respuesta</t>
+        </is>
+      </c>
+      <c r="G435" s="13" t="inlineStr">
+        <is>
+          <t>Dado un ticket con SLA en horas por prioridad
+Entonces el sistema avisa antes de vencer y al vencer</t>
+        </is>
+      </c>
+    </row>
+    <row r="436">
+      <c r="A436" s="12" t="inlineStr">
+        <is>
+          <t>HU-219</t>
+        </is>
+      </c>
+      <c r="B436" s="13" t="inlineStr">
+        <is>
+          <t>Comunicar novedades con campañas segmentadas</t>
+        </is>
+      </c>
+      <c r="C436" s="12" t="inlineStr">
+        <is>
+          <t>EP-21</t>
+        </is>
+      </c>
+      <c r="D436" s="12" t="inlineStr">
+        <is>
+          <t>Sprint 5</t>
+        </is>
+      </c>
+      <c r="E436" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="F436" s="13" t="inlineStr">
+        <is>
+          <t>Audiencia</t>
+        </is>
+      </c>
+      <c r="G436" s="13" t="inlineStr">
+        <is>
+          <t>Cuando defino una campaña con condiciones de audiencia
+Entonces solo la reciben los usuarios que las cumplen</t>
+        </is>
+      </c>
+    </row>
+    <row r="437">
+      <c r="A437" s="12" t="inlineStr">
+        <is>
+          <t>HU-219</t>
+        </is>
+      </c>
+      <c r="B437" s="13" t="inlineStr">
+        <is>
+          <t>Comunicar novedades con campañas segmentadas</t>
+        </is>
+      </c>
+      <c r="C437" s="12" t="inlineStr">
+        <is>
+          <t>EP-21</t>
+        </is>
+      </c>
+      <c r="D437" s="12" t="inlineStr">
+        <is>
+          <t>Sprint 5</t>
+        </is>
+      </c>
+      <c r="E437" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="F437" s="13" t="inlineStr">
+        <is>
+          <t>Entrega</t>
+        </is>
+      </c>
+      <c r="G437" s="13" t="inlineStr">
+        <is>
+          <t>Cuando la campaña está activa
+Entonces el usuario la ve como banner, modal o tarjeta y en la campana</t>
+        </is>
+      </c>
+    </row>
+    <row r="438">
+      <c r="A438" s="12" t="inlineStr">
+        <is>
+          <t>HU-220</t>
+        </is>
+      </c>
+      <c r="B438" s="13" t="inlineStr">
+        <is>
+          <t>Recorrer y operar la bodega en 3D (SIGMA Twin)</t>
+        </is>
+      </c>
+      <c r="C438" s="12" t="inlineStr">
+        <is>
+          <t>EP-06</t>
+        </is>
+      </c>
+      <c r="D438" s="12" t="inlineStr">
+        <is>
+          <t>Sprint 5</t>
+        </is>
+      </c>
+      <c r="E438" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="F438" s="13" t="inlineStr">
+        <is>
+          <t>Mapa de la bodega</t>
+        </is>
+      </c>
+      <c r="G438" s="13" t="inlineStr">
+        <is>
+          <t>Cuando abro SIGMA Twin
+Entonces veo los racks, las cajas por tipo de repuesto y las alertas de stock bajo el mínimo</t>
+        </is>
+      </c>
+    </row>
+    <row r="439">
+      <c r="A439" s="12" t="inlineStr">
+        <is>
+          <t>HU-220</t>
+        </is>
+      </c>
+      <c r="B439" s="13" t="inlineStr">
+        <is>
+          <t>Recorrer y operar la bodega en 3D (SIGMA Twin)</t>
+        </is>
+      </c>
+      <c r="C439" s="12" t="inlineStr">
+        <is>
+          <t>EP-06</t>
+        </is>
+      </c>
+      <c r="D439" s="12" t="inlineStr">
+        <is>
+          <t>Sprint 5</t>
+        </is>
+      </c>
+      <c r="E439" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="F439" s="13" t="inlineStr">
+        <is>
+          <t>Picking</t>
+        </is>
+      </c>
+      <c r="G439" s="13" t="inlineStr">
+        <is>
+          <t>Cuando agrego cajas al picking
+Entonces se respeta el método de salida de la bodega (FEFO, FIFO o LIFO)</t>
+        </is>
+      </c>
+    </row>
+    <row r="440">
+      <c r="A440" s="12" t="inlineStr">
+        <is>
+          <t>HU-220</t>
+        </is>
+      </c>
+      <c r="B440" s="13" t="inlineStr">
+        <is>
+          <t>Recorrer y operar la bodega en 3D (SIGMA Twin)</t>
+        </is>
+      </c>
+      <c r="C440" s="12" t="inlineStr">
+        <is>
+          <t>EP-06</t>
+        </is>
+      </c>
+      <c r="D440" s="12" t="inlineStr">
+        <is>
+          <t>Sprint 5</t>
+        </is>
+      </c>
+      <c r="E440" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="F440" s="13" t="inlineStr">
+        <is>
+          <t>Conteo cíclico</t>
+        </is>
+      </c>
+      <c r="G440" s="13" t="inlineStr">
+        <is>
+          <t>Cuando cuento desde el recorrido
+Entonces queda la exactitud del conteo y las diferencias por caja</t>
+        </is>
+      </c>
+    </row>
+    <row r="441">
+      <c r="A441" s="12" t="inlineStr">
+        <is>
+          <t>HU-221</t>
+        </is>
+      </c>
+      <c r="B441" s="13" t="inlineStr">
+        <is>
+          <t>Ver mi inicio con accesos, alertas y SIGMA AI</t>
+        </is>
+      </c>
+      <c r="C441" s="12" t="inlineStr">
+        <is>
+          <t>EP-18</t>
+        </is>
+      </c>
+      <c r="D441" s="12" t="inlineStr">
+        <is>
+          <t>Sprint 5</t>
+        </is>
+      </c>
+      <c r="E441" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="F441" s="13" t="inlineStr">
+        <is>
+          <t>Accesos por persona</t>
+        </is>
+      </c>
+      <c r="G441" s="13" t="inlineStr">
+        <is>
+          <t>Cuando entro a SIGMA
+Entonces veo mis accesos directos, solo de módulos para los que tengo permiso</t>
+        </is>
+      </c>
+    </row>
+    <row r="442">
+      <c r="A442" s="12" t="inlineStr">
+        <is>
+          <t>HU-221</t>
+        </is>
+      </c>
+      <c r="B442" s="13" t="inlineStr">
+        <is>
+          <t>Ver mi inicio con accesos, alertas y SIGMA AI</t>
+        </is>
+      </c>
+      <c r="C442" s="12" t="inlineStr">
+        <is>
+          <t>EP-18</t>
+        </is>
+      </c>
+      <c r="D442" s="12" t="inlineStr">
+        <is>
+          <t>Sprint 5</t>
+        </is>
+      </c>
+      <c r="E442" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="F442" s="13" t="inlineStr">
+        <is>
+          <t>Requiere atención</t>
+        </is>
+      </c>
+      <c r="G442" s="13" t="inlineStr">
+        <is>
+          <t>Cuando hay alertas, predicciones o OT vencidas
+Entonces aparecen agrupadas en «Requieren tu atención» y se actualizan cada 30 segundos</t>
         </is>
       </c>
     </row>
@@ -50111,11 +52121,11 @@
         </is>
       </c>
       <c r="D10" s="9">
-        <f>SUM('Sprint 5'!$I$6:$I$19)</f>
+        <f>SUM('Sprint 5'!$I$6:$I$31)</f>
         <v/>
       </c>
       <c r="E10" s="9">
-        <f>SUM('Sprint 5'!$O$6:$O$19)</f>
+        <f>SUM('Sprint 5'!$O$6:$O$31)</f>
         <v/>
       </c>
       <c r="F10" s="11">
@@ -50123,11 +52133,11 @@
         <v/>
       </c>
       <c r="G10" s="9">
-        <f>COUNTA('Sprint 5'!$A$6:$A$19)</f>
+        <f>COUNTA('Sprint 5'!$A$6:$A$31)</f>
         <v/>
       </c>
       <c r="H10" s="9">
-        <f>COUNTIF('Sprint 5'!$M$6:$M$19,"Terminada")</f>
+        <f>COUNTIF('Sprint 5'!$M$6:$M$31,"Terminada")</f>
         <v/>
       </c>
       <c r="I10" s="9">
@@ -50460,11 +52470,11 @@
         </is>
       </c>
       <c r="F6" s="12">
-        <f>COUNTIF('Backlog completo'!$L$6:$L$143,$A6)</f>
+        <f>COUNTIF('Backlog completo'!$L$6:$L$155,$A6)</f>
         <v/>
       </c>
       <c r="G6" s="12">
-        <f>SUMIF('Backlog completo'!$L$6:$L$143,$A6,'Backlog completo'!$J$6:$J$143)</f>
+        <f>SUMIF('Backlog completo'!$L$6:$L$155,$A6,'Backlog completo'!$J$6:$J$155)</f>
         <v/>
       </c>
     </row>
@@ -50495,11 +52505,11 @@
         </is>
       </c>
       <c r="F7" s="9">
-        <f>COUNTIF('Backlog completo'!$L$6:$L$143,$A7)</f>
+        <f>COUNTIF('Backlog completo'!$L$6:$L$155,$A7)</f>
         <v/>
       </c>
       <c r="G7" s="9">
-        <f>SUMIF('Backlog completo'!$L$6:$L$143,$A7,'Backlog completo'!$J$6:$J$143)</f>
+        <f>SUMIF('Backlog completo'!$L$6:$L$155,$A7,'Backlog completo'!$J$6:$J$155)</f>
         <v/>
       </c>
     </row>
@@ -50530,11 +52540,11 @@
         </is>
       </c>
       <c r="F8" s="12">
-        <f>COUNTIF('Backlog completo'!$L$6:$L$143,$A8)</f>
+        <f>COUNTIF('Backlog completo'!$L$6:$L$155,$A8)</f>
         <v/>
       </c>
       <c r="G8" s="12">
-        <f>SUMIF('Backlog completo'!$L$6:$L$143,$A8,'Backlog completo'!$J$6:$J$143)</f>
+        <f>SUMIF('Backlog completo'!$L$6:$L$155,$A8,'Backlog completo'!$J$6:$J$155)</f>
         <v/>
       </c>
     </row>
@@ -50565,11 +52575,11 @@
         </is>
       </c>
       <c r="F9" s="9">
-        <f>COUNTIF('Backlog completo'!$L$6:$L$143,$A9)</f>
+        <f>COUNTIF('Backlog completo'!$L$6:$L$155,$A9)</f>
         <v/>
       </c>
       <c r="G9" s="9">
-        <f>SUMIF('Backlog completo'!$L$6:$L$143,$A9,'Backlog completo'!$J$6:$J$143)</f>
+        <f>SUMIF('Backlog completo'!$L$6:$L$155,$A9,'Backlog completo'!$J$6:$J$155)</f>
         <v/>
       </c>
     </row>
@@ -50596,15 +52606,15 @@
       </c>
       <c r="E10" s="13" t="inlineStr">
         <is>
-          <t>Órdenes de trabajo, fallas, bitácora y evidencias en la web. La ejecución en terreno, sin conexión y por voz pasa al Sprint 6.</t>
+          <t>Órdenes de trabajo, fallas, bitácora y evidencias en la web; centro comercial, cobros y procesos automáticos; soporte; SIGMA Twin; carga de datos.</t>
         </is>
       </c>
       <c r="F10" s="12">
-        <f>COUNTIF('Backlog completo'!$L$6:$L$143,$A10)</f>
+        <f>COUNTIF('Backlog completo'!$L$6:$L$155,$A10)</f>
         <v/>
       </c>
       <c r="G10" s="12">
-        <f>SUMIF('Backlog completo'!$L$6:$L$143,$A10,'Backlog completo'!$J$6:$J$143)</f>
+        <f>SUMIF('Backlog completo'!$L$6:$L$155,$A10,'Backlog completo'!$J$6:$J$155)</f>
         <v/>
       </c>
     </row>
@@ -50635,11 +52645,11 @@
         </is>
       </c>
       <c r="F11" s="9">
-        <f>COUNTIF('Backlog completo'!$L$6:$L$143,$A11)</f>
+        <f>COUNTIF('Backlog completo'!$L$6:$L$155,$A11)</f>
         <v/>
       </c>
       <c r="G11" s="9">
-        <f>SUMIF('Backlog completo'!$L$6:$L$143,$A11,'Backlog completo'!$J$6:$J$143)</f>
+        <f>SUMIF('Backlog completo'!$L$6:$L$155,$A11,'Backlog completo'!$J$6:$J$155)</f>
         <v/>
       </c>
     </row>
@@ -50720,7 +52730,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H26"/>
+  <dimension ref="A1:H27"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" style="26" min="1" max="1"/>
@@ -50742,7 +52752,7 @@
     <row r="2" ht="15.75" customHeight="1" s="26">
       <c r="A2" s="28" t="inlineStr">
         <is>
-          <t>20 épicas · objetivo, volumen y Sprint principal</t>
+          <t>21 épicas · objetivo, volumen y Sprint principal</t>
         </is>
       </c>
     </row>
@@ -50805,15 +52815,15 @@
         </is>
       </c>
       <c r="D6" s="9">
-        <f>COUNTIF('Backlog completo'!$B$6:$B$143,$A6)</f>
+        <f>COUNTIF('Backlog completo'!$B$6:$B$155,$A6)</f>
         <v/>
       </c>
       <c r="E6" s="9">
-        <f>SUMIF('Backlog completo'!$B$6:$B$143,$A6,'Backlog completo'!$J$6:$J$143)</f>
+        <f>SUMIF('Backlog completo'!$B$6:$B$155,$A6,'Backlog completo'!$J$6:$J$155)</f>
         <v/>
       </c>
       <c r="F6" s="9">
-        <f>IFERROR(ROUND(AVERAGEIF('Backlog completo'!$B$6:$B$143,$A6,'Backlog completo'!$I$6:$I$143),0),0)</f>
+        <f>IFERROR(ROUND(AVERAGEIF('Backlog completo'!$B$6:$B$155,$A6,'Backlog completo'!$I$6:$I$155),0),0)</f>
         <v/>
       </c>
       <c r="G6" s="9" t="inlineStr">
@@ -50822,7 +52832,7 @@
         </is>
       </c>
       <c r="H6" s="11">
-        <f>IFERROR($E6/SUM($E$6:$E$25),0)</f>
+        <f>IFERROR($E6/SUM($E$6:$E$26),0)</f>
         <v/>
       </c>
     </row>
@@ -50843,15 +52853,15 @@
         </is>
       </c>
       <c r="D7" s="12">
-        <f>COUNTIF('Backlog completo'!$B$6:$B$143,$A7)</f>
+        <f>COUNTIF('Backlog completo'!$B$6:$B$155,$A7)</f>
         <v/>
       </c>
       <c r="E7" s="12">
-        <f>SUMIF('Backlog completo'!$B$6:$B$143,$A7,'Backlog completo'!$J$6:$J$143)</f>
+        <f>SUMIF('Backlog completo'!$B$6:$B$155,$A7,'Backlog completo'!$J$6:$J$155)</f>
         <v/>
       </c>
       <c r="F7" s="12">
-        <f>IFERROR(ROUND(AVERAGEIF('Backlog completo'!$B$6:$B$143,$A7,'Backlog completo'!$I$6:$I$143),0),0)</f>
+        <f>IFERROR(ROUND(AVERAGEIF('Backlog completo'!$B$6:$B$155,$A7,'Backlog completo'!$I$6:$I$155),0),0)</f>
         <v/>
       </c>
       <c r="G7" s="12" t="inlineStr">
@@ -50860,7 +52870,7 @@
         </is>
       </c>
       <c r="H7" s="14">
-        <f>IFERROR($E7/SUM($E$6:$E$25),0)</f>
+        <f>IFERROR($E7/SUM($E$6:$E$26),0)</f>
         <v/>
       </c>
     </row>
@@ -50881,15 +52891,15 @@
         </is>
       </c>
       <c r="D8" s="9">
-        <f>COUNTIF('Backlog completo'!$B$6:$B$143,$A8)</f>
+        <f>COUNTIF('Backlog completo'!$B$6:$B$155,$A8)</f>
         <v/>
       </c>
       <c r="E8" s="9">
-        <f>SUMIF('Backlog completo'!$B$6:$B$143,$A8,'Backlog completo'!$J$6:$J$143)</f>
+        <f>SUMIF('Backlog completo'!$B$6:$B$155,$A8,'Backlog completo'!$J$6:$J$155)</f>
         <v/>
       </c>
       <c r="F8" s="9">
-        <f>IFERROR(ROUND(AVERAGEIF('Backlog completo'!$B$6:$B$143,$A8,'Backlog completo'!$I$6:$I$143),0),0)</f>
+        <f>IFERROR(ROUND(AVERAGEIF('Backlog completo'!$B$6:$B$155,$A8,'Backlog completo'!$I$6:$I$155),0),0)</f>
         <v/>
       </c>
       <c r="G8" s="9" t="inlineStr">
@@ -50898,7 +52908,7 @@
         </is>
       </c>
       <c r="H8" s="11">
-        <f>IFERROR($E8/SUM($E$6:$E$25),0)</f>
+        <f>IFERROR($E8/SUM($E$6:$E$26),0)</f>
         <v/>
       </c>
     </row>
@@ -50919,15 +52929,15 @@
         </is>
       </c>
       <c r="D9" s="12">
-        <f>COUNTIF('Backlog completo'!$B$6:$B$143,$A9)</f>
+        <f>COUNTIF('Backlog completo'!$B$6:$B$155,$A9)</f>
         <v/>
       </c>
       <c r="E9" s="12">
-        <f>SUMIF('Backlog completo'!$B$6:$B$143,$A9,'Backlog completo'!$J$6:$J$143)</f>
+        <f>SUMIF('Backlog completo'!$B$6:$B$155,$A9,'Backlog completo'!$J$6:$J$155)</f>
         <v/>
       </c>
       <c r="F9" s="12">
-        <f>IFERROR(ROUND(AVERAGEIF('Backlog completo'!$B$6:$B$143,$A9,'Backlog completo'!$I$6:$I$143),0),0)</f>
+        <f>IFERROR(ROUND(AVERAGEIF('Backlog completo'!$B$6:$B$155,$A9,'Backlog completo'!$I$6:$I$155),0),0)</f>
         <v/>
       </c>
       <c r="G9" s="12" t="inlineStr">
@@ -50936,7 +52946,7 @@
         </is>
       </c>
       <c r="H9" s="14">
-        <f>IFERROR($E9/SUM($E$6:$E$25),0)</f>
+        <f>IFERROR($E9/SUM($E$6:$E$26),0)</f>
         <v/>
       </c>
     </row>
@@ -50957,15 +52967,15 @@
         </is>
       </c>
       <c r="D10" s="9">
-        <f>COUNTIF('Backlog completo'!$B$6:$B$143,$A10)</f>
+        <f>COUNTIF('Backlog completo'!$B$6:$B$155,$A10)</f>
         <v/>
       </c>
       <c r="E10" s="9">
-        <f>SUMIF('Backlog completo'!$B$6:$B$143,$A10,'Backlog completo'!$J$6:$J$143)</f>
+        <f>SUMIF('Backlog completo'!$B$6:$B$155,$A10,'Backlog completo'!$J$6:$J$155)</f>
         <v/>
       </c>
       <c r="F10" s="9">
-        <f>IFERROR(ROUND(AVERAGEIF('Backlog completo'!$B$6:$B$143,$A10,'Backlog completo'!$I$6:$I$143),0),0)</f>
+        <f>IFERROR(ROUND(AVERAGEIF('Backlog completo'!$B$6:$B$155,$A10,'Backlog completo'!$I$6:$I$155),0),0)</f>
         <v/>
       </c>
       <c r="G10" s="9" t="inlineStr">
@@ -50974,7 +52984,7 @@
         </is>
       </c>
       <c r="H10" s="11">
-        <f>IFERROR($E10/SUM($E$6:$E$25),0)</f>
+        <f>IFERROR($E10/SUM($E$6:$E$26),0)</f>
         <v/>
       </c>
     </row>
@@ -50995,15 +53005,15 @@
         </is>
       </c>
       <c r="D11" s="12">
-        <f>COUNTIF('Backlog completo'!$B$6:$B$143,$A11)</f>
+        <f>COUNTIF('Backlog completo'!$B$6:$B$155,$A11)</f>
         <v/>
       </c>
       <c r="E11" s="12">
-        <f>SUMIF('Backlog completo'!$B$6:$B$143,$A11,'Backlog completo'!$J$6:$J$143)</f>
+        <f>SUMIF('Backlog completo'!$B$6:$B$155,$A11,'Backlog completo'!$J$6:$J$155)</f>
         <v/>
       </c>
       <c r="F11" s="12">
-        <f>IFERROR(ROUND(AVERAGEIF('Backlog completo'!$B$6:$B$143,$A11,'Backlog completo'!$I$6:$I$143),0),0)</f>
+        <f>IFERROR(ROUND(AVERAGEIF('Backlog completo'!$B$6:$B$155,$A11,'Backlog completo'!$I$6:$I$155),0),0)</f>
         <v/>
       </c>
       <c r="G11" s="12" t="inlineStr">
@@ -51012,7 +53022,7 @@
         </is>
       </c>
       <c r="H11" s="14">
-        <f>IFERROR($E11/SUM($E$6:$E$25),0)</f>
+        <f>IFERROR($E11/SUM($E$6:$E$26),0)</f>
         <v/>
       </c>
     </row>
@@ -51033,15 +53043,15 @@
         </is>
       </c>
       <c r="D12" s="9">
-        <f>COUNTIF('Backlog completo'!$B$6:$B$143,$A12)</f>
+        <f>COUNTIF('Backlog completo'!$B$6:$B$155,$A12)</f>
         <v/>
       </c>
       <c r="E12" s="9">
-        <f>SUMIF('Backlog completo'!$B$6:$B$143,$A12,'Backlog completo'!$J$6:$J$143)</f>
+        <f>SUMIF('Backlog completo'!$B$6:$B$155,$A12,'Backlog completo'!$J$6:$J$155)</f>
         <v/>
       </c>
       <c r="F12" s="9">
-        <f>IFERROR(ROUND(AVERAGEIF('Backlog completo'!$B$6:$B$143,$A12,'Backlog completo'!$I$6:$I$143),0),0)</f>
+        <f>IFERROR(ROUND(AVERAGEIF('Backlog completo'!$B$6:$B$155,$A12,'Backlog completo'!$I$6:$I$155),0),0)</f>
         <v/>
       </c>
       <c r="G12" s="9" t="inlineStr">
@@ -51050,7 +53060,7 @@
         </is>
       </c>
       <c r="H12" s="11">
-        <f>IFERROR($E12/SUM($E$6:$E$25),0)</f>
+        <f>IFERROR($E12/SUM($E$6:$E$26),0)</f>
         <v/>
       </c>
     </row>
@@ -51071,15 +53081,15 @@
         </is>
       </c>
       <c r="D13" s="12">
-        <f>COUNTIF('Backlog completo'!$B$6:$B$143,$A13)</f>
+        <f>COUNTIF('Backlog completo'!$B$6:$B$155,$A13)</f>
         <v/>
       </c>
       <c r="E13" s="12">
-        <f>SUMIF('Backlog completo'!$B$6:$B$143,$A13,'Backlog completo'!$J$6:$J$143)</f>
+        <f>SUMIF('Backlog completo'!$B$6:$B$155,$A13,'Backlog completo'!$J$6:$J$155)</f>
         <v/>
       </c>
       <c r="F13" s="12">
-        <f>IFERROR(ROUND(AVERAGEIF('Backlog completo'!$B$6:$B$143,$A13,'Backlog completo'!$I$6:$I$143),0),0)</f>
+        <f>IFERROR(ROUND(AVERAGEIF('Backlog completo'!$B$6:$B$155,$A13,'Backlog completo'!$I$6:$I$155),0),0)</f>
         <v/>
       </c>
       <c r="G13" s="12" t="inlineStr">
@@ -51088,7 +53098,7 @@
         </is>
       </c>
       <c r="H13" s="14">
-        <f>IFERROR($E13/SUM($E$6:$E$25),0)</f>
+        <f>IFERROR($E13/SUM($E$6:$E$26),0)</f>
         <v/>
       </c>
     </row>
@@ -51109,15 +53119,15 @@
         </is>
       </c>
       <c r="D14" s="9">
-        <f>COUNTIF('Backlog completo'!$B$6:$B$143,$A14)</f>
+        <f>COUNTIF('Backlog completo'!$B$6:$B$155,$A14)</f>
         <v/>
       </c>
       <c r="E14" s="9">
-        <f>SUMIF('Backlog completo'!$B$6:$B$143,$A14,'Backlog completo'!$J$6:$J$143)</f>
+        <f>SUMIF('Backlog completo'!$B$6:$B$155,$A14,'Backlog completo'!$J$6:$J$155)</f>
         <v/>
       </c>
       <c r="F14" s="9">
-        <f>IFERROR(ROUND(AVERAGEIF('Backlog completo'!$B$6:$B$143,$A14,'Backlog completo'!$I$6:$I$143),0),0)</f>
+        <f>IFERROR(ROUND(AVERAGEIF('Backlog completo'!$B$6:$B$155,$A14,'Backlog completo'!$I$6:$I$155),0),0)</f>
         <v/>
       </c>
       <c r="G14" s="9" t="inlineStr">
@@ -51126,7 +53136,7 @@
         </is>
       </c>
       <c r="H14" s="11">
-        <f>IFERROR($E14/SUM($E$6:$E$25),0)</f>
+        <f>IFERROR($E14/SUM($E$6:$E$26),0)</f>
         <v/>
       </c>
     </row>
@@ -51147,15 +53157,15 @@
         </is>
       </c>
       <c r="D15" s="12">
-        <f>COUNTIF('Backlog completo'!$B$6:$B$143,$A15)</f>
+        <f>COUNTIF('Backlog completo'!$B$6:$B$155,$A15)</f>
         <v/>
       </c>
       <c r="E15" s="12">
-        <f>SUMIF('Backlog completo'!$B$6:$B$143,$A15,'Backlog completo'!$J$6:$J$143)</f>
+        <f>SUMIF('Backlog completo'!$B$6:$B$155,$A15,'Backlog completo'!$J$6:$J$155)</f>
         <v/>
       </c>
       <c r="F15" s="12">
-        <f>IFERROR(ROUND(AVERAGEIF('Backlog completo'!$B$6:$B$143,$A15,'Backlog completo'!$I$6:$I$143),0),0)</f>
+        <f>IFERROR(ROUND(AVERAGEIF('Backlog completo'!$B$6:$B$155,$A15,'Backlog completo'!$I$6:$I$155),0),0)</f>
         <v/>
       </c>
       <c r="G15" s="12" t="inlineStr">
@@ -51164,7 +53174,7 @@
         </is>
       </c>
       <c r="H15" s="14">
-        <f>IFERROR($E15/SUM($E$6:$E$25),0)</f>
+        <f>IFERROR($E15/SUM($E$6:$E$26),0)</f>
         <v/>
       </c>
     </row>
@@ -51185,15 +53195,15 @@
         </is>
       </c>
       <c r="D16" s="9">
-        <f>COUNTIF('Backlog completo'!$B$6:$B$143,$A16)</f>
+        <f>COUNTIF('Backlog completo'!$B$6:$B$155,$A16)</f>
         <v/>
       </c>
       <c r="E16" s="9">
-        <f>SUMIF('Backlog completo'!$B$6:$B$143,$A16,'Backlog completo'!$J$6:$J$143)</f>
+        <f>SUMIF('Backlog completo'!$B$6:$B$155,$A16,'Backlog completo'!$J$6:$J$155)</f>
         <v/>
       </c>
       <c r="F16" s="9">
-        <f>IFERROR(ROUND(AVERAGEIF('Backlog completo'!$B$6:$B$143,$A16,'Backlog completo'!$I$6:$I$143),0),0)</f>
+        <f>IFERROR(ROUND(AVERAGEIF('Backlog completo'!$B$6:$B$155,$A16,'Backlog completo'!$I$6:$I$155),0),0)</f>
         <v/>
       </c>
       <c r="G16" s="9" t="inlineStr">
@@ -51202,7 +53212,7 @@
         </is>
       </c>
       <c r="H16" s="11">
-        <f>IFERROR($E16/SUM($E$6:$E$25),0)</f>
+        <f>IFERROR($E16/SUM($E$6:$E$26),0)</f>
         <v/>
       </c>
     </row>
@@ -51223,15 +53233,15 @@
         </is>
       </c>
       <c r="D17" s="12">
-        <f>COUNTIF('Backlog completo'!$B$6:$B$143,$A17)</f>
+        <f>COUNTIF('Backlog completo'!$B$6:$B$155,$A17)</f>
         <v/>
       </c>
       <c r="E17" s="12">
-        <f>SUMIF('Backlog completo'!$B$6:$B$143,$A17,'Backlog completo'!$J$6:$J$143)</f>
+        <f>SUMIF('Backlog completo'!$B$6:$B$155,$A17,'Backlog completo'!$J$6:$J$155)</f>
         <v/>
       </c>
       <c r="F17" s="12">
-        <f>IFERROR(ROUND(AVERAGEIF('Backlog completo'!$B$6:$B$143,$A17,'Backlog completo'!$I$6:$I$143),0),0)</f>
+        <f>IFERROR(ROUND(AVERAGEIF('Backlog completo'!$B$6:$B$155,$A17,'Backlog completo'!$I$6:$I$155),0),0)</f>
         <v/>
       </c>
       <c r="G17" s="12" t="inlineStr">
@@ -51240,7 +53250,7 @@
         </is>
       </c>
       <c r="H17" s="14">
-        <f>IFERROR($E17/SUM($E$6:$E$25),0)</f>
+        <f>IFERROR($E17/SUM($E$6:$E$26),0)</f>
         <v/>
       </c>
     </row>
@@ -51261,15 +53271,15 @@
         </is>
       </c>
       <c r="D18" s="9">
-        <f>COUNTIF('Backlog completo'!$B$6:$B$143,$A18)</f>
+        <f>COUNTIF('Backlog completo'!$B$6:$B$155,$A18)</f>
         <v/>
       </c>
       <c r="E18" s="9">
-        <f>SUMIF('Backlog completo'!$B$6:$B$143,$A18,'Backlog completo'!$J$6:$J$143)</f>
+        <f>SUMIF('Backlog completo'!$B$6:$B$155,$A18,'Backlog completo'!$J$6:$J$155)</f>
         <v/>
       </c>
       <c r="F18" s="9">
-        <f>IFERROR(ROUND(AVERAGEIF('Backlog completo'!$B$6:$B$143,$A18,'Backlog completo'!$I$6:$I$143),0),0)</f>
+        <f>IFERROR(ROUND(AVERAGEIF('Backlog completo'!$B$6:$B$155,$A18,'Backlog completo'!$I$6:$I$155),0),0)</f>
         <v/>
       </c>
       <c r="G18" s="9" t="inlineStr">
@@ -51278,7 +53288,7 @@
         </is>
       </c>
       <c r="H18" s="11">
-        <f>IFERROR($E18/SUM($E$6:$E$25),0)</f>
+        <f>IFERROR($E18/SUM($E$6:$E$26),0)</f>
         <v/>
       </c>
     </row>
@@ -51299,15 +53309,15 @@
         </is>
       </c>
       <c r="D19" s="12">
-        <f>COUNTIF('Backlog completo'!$B$6:$B$143,$A19)</f>
+        <f>COUNTIF('Backlog completo'!$B$6:$B$155,$A19)</f>
         <v/>
       </c>
       <c r="E19" s="12">
-        <f>SUMIF('Backlog completo'!$B$6:$B$143,$A19,'Backlog completo'!$J$6:$J$143)</f>
+        <f>SUMIF('Backlog completo'!$B$6:$B$155,$A19,'Backlog completo'!$J$6:$J$155)</f>
         <v/>
       </c>
       <c r="F19" s="12">
-        <f>IFERROR(ROUND(AVERAGEIF('Backlog completo'!$B$6:$B$143,$A19,'Backlog completo'!$I$6:$I$143),0),0)</f>
+        <f>IFERROR(ROUND(AVERAGEIF('Backlog completo'!$B$6:$B$155,$A19,'Backlog completo'!$I$6:$I$155),0),0)</f>
         <v/>
       </c>
       <c r="G19" s="12" t="inlineStr">
@@ -51316,7 +53326,7 @@
         </is>
       </c>
       <c r="H19" s="14">
-        <f>IFERROR($E19/SUM($E$6:$E$25),0)</f>
+        <f>IFERROR($E19/SUM($E$6:$E$26),0)</f>
         <v/>
       </c>
     </row>
@@ -51337,15 +53347,15 @@
         </is>
       </c>
       <c r="D20" s="9">
-        <f>COUNTIF('Backlog completo'!$B$6:$B$143,$A20)</f>
+        <f>COUNTIF('Backlog completo'!$B$6:$B$155,$A20)</f>
         <v/>
       </c>
       <c r="E20" s="9">
-        <f>SUMIF('Backlog completo'!$B$6:$B$143,$A20,'Backlog completo'!$J$6:$J$143)</f>
+        <f>SUMIF('Backlog completo'!$B$6:$B$155,$A20,'Backlog completo'!$J$6:$J$155)</f>
         <v/>
       </c>
       <c r="F20" s="9">
-        <f>IFERROR(ROUND(AVERAGEIF('Backlog completo'!$B$6:$B$143,$A20,'Backlog completo'!$I$6:$I$143),0),0)</f>
+        <f>IFERROR(ROUND(AVERAGEIF('Backlog completo'!$B$6:$B$155,$A20,'Backlog completo'!$I$6:$I$155),0),0)</f>
         <v/>
       </c>
       <c r="G20" s="9" t="inlineStr">
@@ -51354,7 +53364,7 @@
         </is>
       </c>
       <c r="H20" s="11">
-        <f>IFERROR($E20/SUM($E$6:$E$25),0)</f>
+        <f>IFERROR($E20/SUM($E$6:$E$26),0)</f>
         <v/>
       </c>
     </row>
@@ -51375,15 +53385,15 @@
         </is>
       </c>
       <c r="D21" s="12">
-        <f>COUNTIF('Backlog completo'!$B$6:$B$143,$A21)</f>
+        <f>COUNTIF('Backlog completo'!$B$6:$B$155,$A21)</f>
         <v/>
       </c>
       <c r="E21" s="12">
-        <f>SUMIF('Backlog completo'!$B$6:$B$143,$A21,'Backlog completo'!$J$6:$J$143)</f>
+        <f>SUMIF('Backlog completo'!$B$6:$B$155,$A21,'Backlog completo'!$J$6:$J$155)</f>
         <v/>
       </c>
       <c r="F21" s="12">
-        <f>IFERROR(ROUND(AVERAGEIF('Backlog completo'!$B$6:$B$143,$A21,'Backlog completo'!$I$6:$I$143),0),0)</f>
+        <f>IFERROR(ROUND(AVERAGEIF('Backlog completo'!$B$6:$B$155,$A21,'Backlog completo'!$I$6:$I$155),0),0)</f>
         <v/>
       </c>
       <c r="G21" s="12" t="inlineStr">
@@ -51392,7 +53402,7 @@
         </is>
       </c>
       <c r="H21" s="14">
-        <f>IFERROR($E21/SUM($E$6:$E$25),0)</f>
+        <f>IFERROR($E21/SUM($E$6:$E$26),0)</f>
         <v/>
       </c>
     </row>
@@ -51413,15 +53423,15 @@
         </is>
       </c>
       <c r="D22" s="9">
-        <f>COUNTIF('Backlog completo'!$B$6:$B$143,$A22)</f>
+        <f>COUNTIF('Backlog completo'!$B$6:$B$155,$A22)</f>
         <v/>
       </c>
       <c r="E22" s="9">
-        <f>SUMIF('Backlog completo'!$B$6:$B$143,$A22,'Backlog completo'!$J$6:$J$143)</f>
+        <f>SUMIF('Backlog completo'!$B$6:$B$155,$A22,'Backlog completo'!$J$6:$J$155)</f>
         <v/>
       </c>
       <c r="F22" s="9">
-        <f>IFERROR(ROUND(AVERAGEIF('Backlog completo'!$B$6:$B$143,$A22,'Backlog completo'!$I$6:$I$143),0),0)</f>
+        <f>IFERROR(ROUND(AVERAGEIF('Backlog completo'!$B$6:$B$155,$A22,'Backlog completo'!$I$6:$I$155),0),0)</f>
         <v/>
       </c>
       <c r="G22" s="9" t="inlineStr">
@@ -51430,7 +53440,7 @@
         </is>
       </c>
       <c r="H22" s="11">
-        <f>IFERROR($E22/SUM($E$6:$E$25),0)</f>
+        <f>IFERROR($E22/SUM($E$6:$E$26),0)</f>
         <v/>
       </c>
     </row>
@@ -51451,15 +53461,15 @@
         </is>
       </c>
       <c r="D23" s="12">
-        <f>COUNTIF('Backlog completo'!$B$6:$B$143,$A23)</f>
+        <f>COUNTIF('Backlog completo'!$B$6:$B$155,$A23)</f>
         <v/>
       </c>
       <c r="E23" s="12">
-        <f>SUMIF('Backlog completo'!$B$6:$B$143,$A23,'Backlog completo'!$J$6:$J$143)</f>
+        <f>SUMIF('Backlog completo'!$B$6:$B$155,$A23,'Backlog completo'!$J$6:$J$155)</f>
         <v/>
       </c>
       <c r="F23" s="12">
-        <f>IFERROR(ROUND(AVERAGEIF('Backlog completo'!$B$6:$B$143,$A23,'Backlog completo'!$I$6:$I$143),0),0)</f>
+        <f>IFERROR(ROUND(AVERAGEIF('Backlog completo'!$B$6:$B$155,$A23,'Backlog completo'!$I$6:$I$155),0),0)</f>
         <v/>
       </c>
       <c r="G23" s="12" t="inlineStr">
@@ -51468,7 +53478,7 @@
         </is>
       </c>
       <c r="H23" s="14">
-        <f>IFERROR($E23/SUM($E$6:$E$25),0)</f>
+        <f>IFERROR($E23/SUM($E$6:$E$26),0)</f>
         <v/>
       </c>
     </row>
@@ -51489,15 +53499,15 @@
         </is>
       </c>
       <c r="D24" s="9">
-        <f>COUNTIF('Backlog completo'!$B$6:$B$143,$A24)</f>
+        <f>COUNTIF('Backlog completo'!$B$6:$B$155,$A24)</f>
         <v/>
       </c>
       <c r="E24" s="9">
-        <f>SUMIF('Backlog completo'!$B$6:$B$143,$A24,'Backlog completo'!$J$6:$J$143)</f>
+        <f>SUMIF('Backlog completo'!$B$6:$B$155,$A24,'Backlog completo'!$J$6:$J$155)</f>
         <v/>
       </c>
       <c r="F24" s="9">
-        <f>IFERROR(ROUND(AVERAGEIF('Backlog completo'!$B$6:$B$143,$A24,'Backlog completo'!$I$6:$I$143),0),0)</f>
+        <f>IFERROR(ROUND(AVERAGEIF('Backlog completo'!$B$6:$B$155,$A24,'Backlog completo'!$I$6:$I$155),0),0)</f>
         <v/>
       </c>
       <c r="G24" s="9" t="inlineStr">
@@ -51506,7 +53516,7 @@
         </is>
       </c>
       <c r="H24" s="11">
-        <f>IFERROR($E24/SUM($E$6:$E$25),0)</f>
+        <f>IFERROR($E24/SUM($E$6:$E$26),0)</f>
         <v/>
       </c>
     </row>
@@ -51527,15 +53537,15 @@
         </is>
       </c>
       <c r="D25" s="12">
-        <f>COUNTIF('Backlog completo'!$B$6:$B$143,$A25)</f>
+        <f>COUNTIF('Backlog completo'!$B$6:$B$155,$A25)</f>
         <v/>
       </c>
       <c r="E25" s="12">
-        <f>SUMIF('Backlog completo'!$B$6:$B$143,$A25,'Backlog completo'!$J$6:$J$143)</f>
+        <f>SUMIF('Backlog completo'!$B$6:$B$155,$A25,'Backlog completo'!$J$6:$J$155)</f>
         <v/>
       </c>
       <c r="F25" s="12">
-        <f>IFERROR(ROUND(AVERAGEIF('Backlog completo'!$B$6:$B$143,$A25,'Backlog completo'!$I$6:$I$143),0),0)</f>
+        <f>IFERROR(ROUND(AVERAGEIF('Backlog completo'!$B$6:$B$155,$A25,'Backlog completo'!$I$6:$I$155),0),0)</f>
         <v/>
       </c>
       <c r="G25" s="12" t="inlineStr">
@@ -51544,30 +53554,68 @@
         </is>
       </c>
       <c r="H25" s="14">
-        <f>IFERROR($E25/SUM($E$6:$E$25),0)</f>
+        <f>IFERROR($E25/SUM($E$6:$E$26),0)</f>
         <v/>
       </c>
     </row>
     <row r="26" ht="15" customHeight="1" s="26">
-      <c r="A26" s="15" t="n"/>
-      <c r="B26" s="16" t="inlineStr">
+      <c r="A26" s="12" t="inlineStr">
+        <is>
+          <t>EP-21</t>
+        </is>
+      </c>
+      <c r="B26" s="13" t="inlineStr">
+        <is>
+          <t>Operación comercial y de plataforma</t>
+        </is>
+      </c>
+      <c r="C26" s="13" t="inlineStr">
+        <is>
+          <t>Vender, cobrar y sostener SIGMA como servicio: del primer contacto a la suscripción pagada, con procesos automáticos, correo confiable y una mesa de ayuda para el cliente.</t>
+        </is>
+      </c>
+      <c r="D26" s="12">
+        <f>COUNTIF('Backlog completo'!$B$6:$B$155,$A26)</f>
+        <v/>
+      </c>
+      <c r="E26" s="12">
+        <f>SUMIF('Backlog completo'!$B$6:$B$155,$A26,'Backlog completo'!$J$6:$J$155)</f>
+        <v/>
+      </c>
+      <c r="F26" s="12">
+        <f>IFERROR(ROUND(AVERAGEIF('Backlog completo'!$B$6:$B$155,$A26,'Backlog completo'!$I$6:$I$155),0),0)</f>
+        <v/>
+      </c>
+      <c r="G26" s="12" t="inlineStr">
+        <is>
+          <t>Sprint 5</t>
+        </is>
+      </c>
+      <c r="H26" s="14">
+        <f>IFERROR($E26/SUM($E$6:$E$26),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="15" t="n"/>
+      <c r="B27" s="16" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="C26" s="16" t="n"/>
-      <c r="D26" s="15">
-        <f>SUM(D6:D25)</f>
+      <c r="C27" s="16" t="n"/>
+      <c r="D27" s="15">
+        <f>SUM(D6:D26)</f>
         <v/>
       </c>
-      <c r="E26" s="15">
-        <f>SUM(E6:E25)</f>
+      <c r="E27" s="15">
+        <f>SUM(E6:E26)</f>
         <v/>
       </c>
-      <c r="F26" s="15" t="n"/>
-      <c r="G26" s="15" t="n"/>
-      <c r="H26" s="17">
-        <f>SUM(H6:H25)</f>
+      <c r="F27" s="15" t="n"/>
+      <c r="G27" s="15" t="n"/>
+      <c r="H27" s="17">
+        <f>SUM(H6:H26)</f>
         <v/>
       </c>
     </row>
@@ -57130,7 +59178,7 @@
       </c>
       <c r="M6" s="9" t="inlineStr">
         <is>
-          <t>En revisión</t>
+          <t>Terminada</t>
         </is>
       </c>
       <c r="N6" s="10" t="inlineStr">
@@ -57201,7 +59249,7 @@
       </c>
       <c r="M7" s="12" t="inlineStr">
         <is>
-          <t>En revisión</t>
+          <t>Terminada</t>
         </is>
       </c>
       <c r="N7" s="13" t="inlineStr">
@@ -57272,7 +59320,7 @@
       </c>
       <c r="M8" s="12" t="inlineStr">
         <is>
-          <t>En revisión</t>
+          <t>Terminada</t>
         </is>
       </c>
       <c r="N8" s="13" t="inlineStr">
@@ -57343,7 +59391,7 @@
       </c>
       <c r="M9" s="9" t="inlineStr">
         <is>
-          <t>En revisión</t>
+          <t>Terminada</t>
         </is>
       </c>
       <c r="N9" s="10" t="inlineStr">
@@ -57414,7 +59462,7 @@
       </c>
       <c r="M10" s="12" t="inlineStr">
         <is>
-          <t>En revisión</t>
+          <t>Terminada</t>
         </is>
       </c>
       <c r="N10" s="13" t="inlineStr">
@@ -57485,7 +59533,7 @@
       </c>
       <c r="M11" s="9" t="inlineStr">
         <is>
-          <t>En revisión</t>
+          <t>Terminada</t>
         </is>
       </c>
       <c r="N11" s="10" t="inlineStr">
@@ -57556,7 +59604,7 @@
       </c>
       <c r="M12" s="12" t="inlineStr">
         <is>
-          <t>En revisión</t>
+          <t>Terminada</t>
         </is>
       </c>
       <c r="N12" s="13" t="inlineStr">
@@ -57627,7 +59675,7 @@
       </c>
       <c r="M13" s="9" t="inlineStr">
         <is>
-          <t>Por hacer</t>
+          <t>Terminada</t>
         </is>
       </c>
       <c r="N13" s="10" t="inlineStr">
@@ -57698,7 +59746,7 @@
       </c>
       <c r="M14" s="12" t="inlineStr">
         <is>
-          <t>En revisión</t>
+          <t>Terminada</t>
         </is>
       </c>
       <c r="N14" s="13" t="inlineStr">
@@ -57769,7 +59817,7 @@
       </c>
       <c r="M15" s="9" t="inlineStr">
         <is>
-          <t>En revisión</t>
+          <t>Terminada</t>
         </is>
       </c>
       <c r="N15" s="10" t="inlineStr">
@@ -57840,7 +59888,7 @@
       </c>
       <c r="M16" s="12" t="inlineStr">
         <is>
-          <t>En revisión</t>
+          <t>Terminada</t>
         </is>
       </c>
       <c r="N16" s="13" t="inlineStr">
@@ -57911,7 +59959,7 @@
       </c>
       <c r="M17" s="9" t="inlineStr">
         <is>
-          <t>En revisión</t>
+          <t>Terminada</t>
         </is>
       </c>
       <c r="N17" s="10" t="inlineStr">
@@ -57982,7 +60030,7 @@
       </c>
       <c r="M18" s="12" t="inlineStr">
         <is>
-          <t>En revisión</t>
+          <t>Terminada</t>
         </is>
       </c>
       <c r="N18" s="13" t="inlineStr">
@@ -58053,7 +60101,7 @@
       </c>
       <c r="M19" s="9" t="inlineStr">
         <is>
-          <t>Por hacer</t>
+          <t>Terminada</t>
         </is>
       </c>
       <c r="N19" s="10" t="inlineStr">
@@ -58124,7 +60172,7 @@
       </c>
       <c r="M20" s="12" t="inlineStr">
         <is>
-          <t>En revisión</t>
+          <t>Terminada</t>
         </is>
       </c>
       <c r="N20" s="13" t="inlineStr">
@@ -58195,7 +60243,7 @@
       </c>
       <c r="M21" s="9" t="inlineStr">
         <is>
-          <t>En revisión</t>
+          <t>Terminada</t>
         </is>
       </c>
       <c r="N21" s="10" t="inlineStr">
@@ -58266,7 +60314,7 @@
       </c>
       <c r="M22" s="12" t="inlineStr">
         <is>
-          <t>Por hacer</t>
+          <t>Terminada</t>
         </is>
       </c>
       <c r="N22" s="13" t="inlineStr">
@@ -58337,7 +60385,7 @@
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
-          <t>En revisión</t>
+          <t>Terminada</t>
         </is>
       </c>
       <c r="N23" s="10" t="inlineStr">
@@ -58408,7 +60456,7 @@
       </c>
       <c r="M24" s="12" t="inlineStr">
         <is>
-          <t>En revisión</t>
+          <t>Terminada</t>
         </is>
       </c>
       <c r="N24" s="13" t="inlineStr">
@@ -58509,7 +60557,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:P20"/>
+  <dimension ref="A1:P32"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" style="26" min="1" max="1"/>
@@ -58550,7 +60598,7 @@
         </is>
       </c>
       <c r="B3" s="20">
-        <f>COUNTA($A$6:$A$19)</f>
+        <f>COUNTA($A$6:$A$31)</f>
         <v/>
       </c>
       <c r="C3" s="19" t="inlineStr">
@@ -58559,7 +60607,7 @@
         </is>
       </c>
       <c r="D3" s="20">
-        <f>SUM($I$6:$I$19)</f>
+        <f>SUM($I$6:$I$31)</f>
         <v/>
       </c>
       <c r="E3" s="19" t="inlineStr">
@@ -58568,7 +60616,7 @@
         </is>
       </c>
       <c r="F3" s="20">
-        <f>SUM($O$6:$O$19)</f>
+        <f>SUM($O$6:$O$31)</f>
         <v/>
       </c>
       <c r="G3" s="19" t="inlineStr">
@@ -58577,7 +60625,7 @@
         </is>
       </c>
       <c r="H3" s="21">
-        <f>IFERROR(SUM($O$6:$O$19)/SUM($I$6:$I$19),0)</f>
+        <f>IFERROR(SUM($O$6:$O$31)/SUM($I$6:$I$31),0)</f>
         <v/>
       </c>
       <c r="I3" s="19" t="inlineStr">
@@ -58586,7 +60634,7 @@
         </is>
       </c>
       <c r="J3" s="20">
-        <f>COUNTIF($M$6:$M$19,"Terminada")</f>
+        <f>COUNTIF($M$6:$M$31,"Terminada")</f>
         <v/>
       </c>
       <c r="K3" s="19" t="inlineStr">
@@ -58738,7 +60786,7 @@
       </c>
       <c r="M6" s="9" t="inlineStr">
         <is>
-          <t>En revisión</t>
+          <t>Terminada</t>
         </is>
       </c>
       <c r="N6" s="10" t="inlineStr">
@@ -58809,7 +60857,7 @@
       </c>
       <c r="M7" s="12" t="inlineStr">
         <is>
-          <t>En revisión</t>
+          <t>Terminada</t>
         </is>
       </c>
       <c r="N7" s="13" t="inlineStr">
@@ -58880,7 +60928,7 @@
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>En revisión</t>
+          <t>Terminada</t>
         </is>
       </c>
       <c r="N8" s="10" t="inlineStr">
@@ -58951,7 +60999,7 @@
       </c>
       <c r="M9" s="9" t="inlineStr">
         <is>
-          <t>En revisión</t>
+          <t>Terminada</t>
         </is>
       </c>
       <c r="N9" s="10" t="inlineStr">
@@ -59022,7 +61070,7 @@
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>En revisión</t>
+          <t>Terminada</t>
         </is>
       </c>
       <c r="N10" s="10" t="inlineStr">
@@ -59164,7 +61212,7 @@
       </c>
       <c r="M12" s="12" t="inlineStr">
         <is>
-          <t>En revisión</t>
+          <t>Terminada</t>
         </is>
       </c>
       <c r="N12" s="13" t="inlineStr">
@@ -59235,7 +61283,7 @@
       </c>
       <c r="M13" s="9" t="inlineStr">
         <is>
-          <t>En revisión</t>
+          <t>Terminada</t>
         </is>
       </c>
       <c r="N13" s="10" t="inlineStr">
@@ -59306,7 +61354,7 @@
       </c>
       <c r="M14" s="9" t="inlineStr">
         <is>
-          <t>En revisión</t>
+          <t>Terminada</t>
         </is>
       </c>
       <c r="N14" s="10" t="inlineStr">
@@ -59377,7 +61425,7 @@
       </c>
       <c r="M15" s="12" t="inlineStr">
         <is>
-          <t>En revisión</t>
+          <t>Terminada</t>
         </is>
       </c>
       <c r="N15" s="13" t="inlineStr">
@@ -59452,7 +61500,7 @@
       </c>
       <c r="M16" s="9" t="inlineStr">
         <is>
-          <t>En revisión</t>
+          <t>Terminada</t>
         </is>
       </c>
       <c r="N16" s="10" t="inlineStr">
@@ -59598,7 +61646,7 @@
       </c>
       <c r="M18" s="9" t="inlineStr">
         <is>
-          <t>Por hacer</t>
+          <t>Terminada</t>
         </is>
       </c>
       <c r="N18" s="10" t="inlineStr">
@@ -59669,7 +61717,7 @@
       </c>
       <c r="M19" s="12" t="inlineStr">
         <is>
-          <t>Por hacer</t>
+          <t>Terminada</t>
         </is>
       </c>
       <c r="N19" s="13" t="inlineStr">
@@ -59684,45 +61732,933 @@
       <c r="P19" s="13" t="n"/>
     </row>
     <row r="20" ht="30" customHeight="1" s="26">
-      <c r="A20" s="15" t="n"/>
-      <c r="B20" s="15" t="n"/>
-      <c r="C20" s="16" t="inlineStr">
+      <c r="A20" s="12" t="inlineStr">
+        <is>
+          <t>HU-210</t>
+        </is>
+      </c>
+      <c r="B20" s="12" t="inlineStr">
+        <is>
+          <t>EP-21</t>
+        </is>
+      </c>
+      <c r="C20" s="13" t="inlineStr">
+        <is>
+          <t>Gestionar los leads en el pipeline comercial</t>
+        </is>
+      </c>
+      <c r="D20" s="13" t="inlineStr">
+        <is>
+          <t>ejecutivo comercial de SIGMA</t>
+        </is>
+      </c>
+      <c r="E20" s="13" t="inlineStr">
+        <is>
+          <t>registrar un lead con su país e identificador y llevarlo por etapas hasta concretarlo</t>
+        </is>
+      </c>
+      <c r="F20" s="13" t="inlineStr">
+        <is>
+          <t>no perder el seguimiento de ningún prospecto y saber cuánto hay en cada etapa</t>
+        </is>
+      </c>
+      <c r="G20" s="12" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="H20" s="12" t="n">
+        <v>90</v>
+      </c>
+      <c r="I20" s="12" t="n">
+        <v>8</v>
+      </c>
+      <c r="J20" s="12" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="K20" s="13" t="inlineStr">
+        <is>
+          <t>HU-190</t>
+        </is>
+      </c>
+      <c r="L20" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="M20" s="12" t="inlineStr">
+        <is>
+          <t>Terminada</t>
+        </is>
+      </c>
+      <c r="N20" s="13" t="inlineStr">
+        <is>
+          <t>Bryan Chávez</t>
+        </is>
+      </c>
+      <c r="O20" s="12">
+        <f>IF($M20="Terminada",$I20,0)</f>
+        <v/>
+      </c>
+      <c r="P20" s="13" t="inlineStr">
+        <is>
+          <t>Centro Comercial V2 (menú Comercial): Resumen, Pipeline, Clientes y Suscripciones, con cajones laterales. Ciclo probado de punta a punta con Hamburgo SA.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="30" customHeight="1" s="26">
+      <c r="A21" s="12" t="inlineStr">
+        <is>
+          <t>HU-211</t>
+        </is>
+      </c>
+      <c r="B21" s="12" t="inlineStr">
+        <is>
+          <t>EP-21</t>
+        </is>
+      </c>
+      <c r="C21" s="13" t="inlineStr">
+        <is>
+          <t>Enviar la propuesta y generar el contrato</t>
+        </is>
+      </c>
+      <c r="D21" s="13" t="inlineStr">
+        <is>
+          <t>ejecutivo comercial de SIGMA</t>
+        </is>
+      </c>
+      <c r="E21" s="13" t="inlineStr">
+        <is>
+          <t>armar una propuesta con plan estándar o personalizado y generar el contrato desde ella</t>
+        </is>
+      </c>
+      <c r="F21" s="13" t="inlineStr">
+        <is>
+          <t>que el cliente reciba una oferta clara y firmable, con sus versiones guardadas</t>
+        </is>
+      </c>
+      <c r="G21" s="12" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="H21" s="12" t="n">
+        <v>90</v>
+      </c>
+      <c r="I21" s="12" t="n">
+        <v>8</v>
+      </c>
+      <c r="J21" s="12" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="K21" s="13" t="inlineStr">
+        <is>
+          <t>HU-210, HU-190</t>
+        </is>
+      </c>
+      <c r="L21" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="M21" s="12" t="inlineStr">
+        <is>
+          <t>Terminada</t>
+        </is>
+      </c>
+      <c r="N21" s="13" t="inlineStr">
+        <is>
+          <t>Bryan Chávez</t>
+        </is>
+      </c>
+      <c r="O21" s="12">
+        <f>IF($M21="Terminada",$I21,0)</f>
+        <v/>
+      </c>
+      <c r="P21" s="13" t="inlineStr">
+        <is>
+          <t>Propuesta con Básico/Medio/Full o plan personalizado, implementación, descuento y vigencia; el contrato congela los números de la propuesta.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="30" customHeight="1" s="26">
+      <c r="A22" s="12" t="inlineStr">
+        <is>
+          <t>HU-212</t>
+        </is>
+      </c>
+      <c r="B22" s="12" t="inlineStr">
+        <is>
+          <t>EP-21</t>
+        </is>
+      </c>
+      <c r="C22" s="13" t="inlineStr">
+        <is>
+          <t>Firmar el contrato en línea</t>
+        </is>
+      </c>
+      <c r="D22" s="13" t="inlineStr">
+        <is>
+          <t>representante del cliente</t>
+        </is>
+      </c>
+      <c r="E22" s="13" t="inlineStr">
+        <is>
+          <t>leer el contrato y firmarlo desde el enlace que recibí por correo, sin crear una cuenta</t>
+        </is>
+      </c>
+      <c r="F22" s="13" t="inlineStr">
+        <is>
+          <t>dejar la contratación cerrada con respaldo legal sin trámites presenciales</t>
+        </is>
+      </c>
+      <c r="G22" s="12" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="H22" s="12" t="n">
+        <v>90</v>
+      </c>
+      <c r="I22" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="J22" s="12" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="K22" s="13" t="inlineStr">
+        <is>
+          <t>HU-211</t>
+        </is>
+      </c>
+      <c r="L22" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="M22" s="12" t="inlineStr">
+        <is>
+          <t>Terminada</t>
+        </is>
+      </c>
+      <c r="N22" s="13" t="inlineStr">
+        <is>
+          <t>Bryan Chávez</t>
+        </is>
+      </c>
+      <c r="O22" s="12">
+        <f>IF($M22="Terminada",$I22,0)</f>
+        <v/>
+      </c>
+      <c r="P22" s="13" t="inlineStr">
+        <is>
+          <t>Firma.aspx es pública; el enlace es de un solo uso por contrato, con hash SHA-256 y registro de fecha e IP.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="30" customHeight="1" s="26">
+      <c r="A23" s="12" t="inlineStr">
+        <is>
+          <t>HU-213</t>
+        </is>
+      </c>
+      <c r="B23" s="12" t="inlineStr">
+        <is>
+          <t>EP-21</t>
+        </is>
+      </c>
+      <c r="C23" s="13" t="inlineStr">
+        <is>
+          <t>Cobrar la suscripción con Webpay o transferencia</t>
+        </is>
+      </c>
+      <c r="D23" s="13" t="inlineStr">
+        <is>
+          <t>administrador de SIGMA</t>
+        </is>
+      </c>
+      <c r="E23" s="13" t="inlineStr">
+        <is>
+          <t>emitir cada período de cobro y registrar su pago por Webpay o por transferencia verificada</t>
+        </is>
+      </c>
+      <c r="F23" s="13" t="inlineStr">
+        <is>
+          <t>saber qué cliente está al día y no perder ningún cobro</t>
+        </is>
+      </c>
+      <c r="G23" s="12" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="H23" s="12" t="n">
+        <v>90</v>
+      </c>
+      <c r="I23" s="12" t="n">
+        <v>8</v>
+      </c>
+      <c r="J23" s="12" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="K23" s="13" t="inlineStr">
+        <is>
+          <t>HU-191, HU-212</t>
+        </is>
+      </c>
+      <c r="L23" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="M23" s="12" t="inlineStr">
+        <is>
+          <t>Terminada</t>
+        </is>
+      </c>
+      <c r="N23" s="13" t="inlineStr">
+        <is>
+          <t>Bryan Chávez</t>
+        </is>
+      </c>
+      <c r="O23" s="12">
+        <f>IF($M23="Terminada",$I23,0)</f>
+        <v/>
+      </c>
+      <c r="P23" s="13" t="inlineStr">
+        <is>
+          <t>Chile: UF a pesos del día (Webpay Plus o transferencia nacional). Exterior: USD por transferencia internacional. Mi suscripción (Renovar.aspx) y Pagar.aspx para el cliente.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="30" customHeight="1" s="26">
+      <c r="A24" s="12" t="inlineStr">
+        <is>
+          <t>HU-214</t>
+        </is>
+      </c>
+      <c r="B24" s="12" t="inlineStr">
+        <is>
+          <t>EP-21</t>
+        </is>
+      </c>
+      <c r="C24" s="13" t="inlineStr">
+        <is>
+          <t>Atender clientes de otros países</t>
+        </is>
+      </c>
+      <c r="D24" s="13" t="inlineStr">
+        <is>
+          <t>administrador de SIGMA</t>
+        </is>
+      </c>
+      <c r="E24" s="13" t="inlineStr">
+        <is>
+          <t>registrar empresas de Chile, Argentina, Colombia, Ecuador, México y Perú con su identificador, zona horaria y moneda</t>
+        </is>
+      </c>
+      <c r="F24" s="13" t="inlineStr">
+        <is>
+          <t>vender SIGMA fuera de Chile sin cambiar el sistema</t>
+        </is>
+      </c>
+      <c r="G24" s="12" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="H24" s="12" t="n">
+        <v>75</v>
+      </c>
+      <c r="I24" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="J24" s="12" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="K24" s="13" t="inlineStr">
+        <is>
+          <t>HU-210</t>
+        </is>
+      </c>
+      <c r="L24" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="M24" s="12" t="inlineStr">
+        <is>
+          <t>Terminada</t>
+        </is>
+      </c>
+      <c r="N24" s="13" t="inlineStr">
+        <is>
+          <t>Bryan Chávez</t>
+        </is>
+      </c>
+      <c r="O24" s="12">
+        <f>IF($M24="Terminada",$I24,0)</f>
+        <v/>
+      </c>
+      <c r="P24" s="13" t="inlineStr">
+        <is>
+          <t>Moneda: Chile en UF cobrado en pesos; el resto en USD. El nombre del identificador y su validación dependen del país.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="30" customHeight="1" s="26">
+      <c r="A25" s="12" t="inlineStr">
+        <is>
+          <t>HU-215</t>
+        </is>
+      </c>
+      <c r="B25" s="12" t="inlineStr">
+        <is>
+          <t>EP-21</t>
+        </is>
+      </c>
+      <c r="C25" s="13" t="inlineStr">
+        <is>
+          <t>Ejecutar los procesos automáticos de SIGMA</t>
+        </is>
+      </c>
+      <c r="D25" s="13" t="inlineStr">
+        <is>
+          <t>administrador de SIGMA</t>
+        </is>
+      </c>
+      <c r="E25" s="13" t="inlineStr">
+        <is>
+          <t>que ocurrencias, órdenes automáticas, cobros, alertas, UF y vencimiento de demos corran solos cada cierto tiempo</t>
+        </is>
+      </c>
+      <c r="F25" s="13" t="inlineStr">
+        <is>
+          <t>no depender de que alguien abra la web ni de un servidor con agendador</t>
+        </is>
+      </c>
+      <c r="G25" s="12" t="inlineStr">
+        <is>
+          <t>Web (infraestructura)</t>
+        </is>
+      </c>
+      <c r="H25" s="12" t="n">
+        <v>90</v>
+      </c>
+      <c r="I25" s="12" t="n">
+        <v>8</v>
+      </c>
+      <c r="J25" s="12" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="K25" s="13" t="inlineStr">
+        <is>
+          <t>HU-094, HU-111</t>
+        </is>
+      </c>
+      <c r="L25" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="M25" s="12" t="inlineStr">
+        <is>
+          <t>Terminada</t>
+        </is>
+      </c>
+      <c r="N25" s="13" t="inlineStr">
+        <is>
+          <t>Bryan Chávez</t>
+        </is>
+      </c>
+      <c r="O25" s="12">
+        <f>IF($M25="Terminada",$I25,0)</f>
+        <v/>
+      </c>
+      <c r="P25" s="13" t="inlineStr">
+        <is>
+          <t>Planificador interno (Timer en Global.asax) más Jobs.aspx con clave; GitHub Actions lo despierta cada 5 minutos (jobs-sigma.yml). Hospedaje sin SQL Agent ni cron.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="30" customHeight="1" s="26">
+      <c r="A26" s="12" t="inlineStr">
+        <is>
+          <t>HU-216</t>
+        </is>
+      </c>
+      <c r="B26" s="12" t="inlineStr">
+        <is>
+          <t>EP-21</t>
+        </is>
+      </c>
+      <c r="C26" s="13" t="inlineStr">
+        <is>
+          <t>Enviar los correos con reintentos y copia de monitoreo</t>
+        </is>
+      </c>
+      <c r="D26" s="13" t="inlineStr">
+        <is>
+          <t>administrador de SIGMA</t>
+        </is>
+      </c>
+      <c r="E26" s="13" t="inlineStr">
+        <is>
+          <t>que todo correo del sistema pase por una cola con reintentos y que yo reciba copia oculta</t>
+        </is>
+      </c>
+      <c r="F26" s="13" t="inlineStr">
+        <is>
+          <t>que un fallo del servidor de correo no pierda mensajes y poder vigilar lo que se envía</t>
+        </is>
+      </c>
+      <c r="G26" s="12" t="inlineStr">
+        <is>
+          <t>Web (infraestructura)</t>
+        </is>
+      </c>
+      <c r="H26" s="12" t="n">
+        <v>80</v>
+      </c>
+      <c r="I26" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="J26" s="12" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="K26" s="13" t="inlineStr">
+        <is>
+          <t>HU-215</t>
+        </is>
+      </c>
+      <c r="L26" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="M26" s="12" t="inlineStr">
+        <is>
+          <t>Terminada</t>
+        </is>
+      </c>
+      <c r="N26" s="13" t="inlineStr">
+        <is>
+          <t>Bryan Chávez</t>
+        </is>
+      </c>
+      <c r="O26" s="12">
+        <f>IF($M26="Terminada",$I26,0)</f>
+        <v/>
+      </c>
+      <c r="P26" s="13" t="inlineStr">
+        <is>
+          <t>Correo_Cola: se envía de inmediato; si falla, el job CORREOS_COLA reintenta hasta 5 veces. CorreoMonitorearA agrega copia oculta sin cambiar los destinatarios reales.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="30" customHeight="1" s="26">
+      <c r="A27" s="12" t="inlineStr">
+        <is>
+          <t>HU-217</t>
+        </is>
+      </c>
+      <c r="B27" s="12" t="inlineStr">
+        <is>
+          <t>EP-21</t>
+        </is>
+      </c>
+      <c r="C27" s="13" t="inlineStr">
+        <is>
+          <t>Reportar un problema y consultar la ayuda de la pantalla</t>
+        </is>
+      </c>
+      <c r="D27" s="13" t="inlineStr">
+        <is>
+          <t>usuario de SIGMA</t>
+        </is>
+      </c>
+      <c r="E27" s="13" t="inlineStr">
+        <is>
+          <t>reportar un problema desde cualquier pantalla y leer la ayuda contextual de esa pantalla</t>
+        </is>
+      </c>
+      <c r="F27" s="13" t="inlineStr">
+        <is>
+          <t>resolver mis dudas sin llamar y que soporte reciba el contexto</t>
+        </is>
+      </c>
+      <c r="G27" s="12" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="H27" s="12" t="n">
+        <v>85</v>
+      </c>
+      <c r="I27" s="12" t="n">
+        <v>8</v>
+      </c>
+      <c r="J27" s="12" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="K27" s="13" t="inlineStr">
+        <is>
+          <t>HU-006</t>
+        </is>
+      </c>
+      <c r="L27" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="M27" s="12" t="inlineStr">
+        <is>
+          <t>Terminada</t>
+        </is>
+      </c>
+      <c r="N27" s="13" t="inlineStr">
+        <is>
+          <t>Bryan Chávez</t>
+        </is>
+      </c>
+      <c r="O27" s="12">
+        <f>IF($M27="Terminada",$I27,0)</f>
+        <v/>
+      </c>
+      <c r="P27" s="13" t="inlineStr">
+        <is>
+          <t>Menú Soporte con 13 pantallas (BD/359–365). «Reportar problema» y «? Ayuda» viven en el master. La ticketera es del plan (cupo mensual).</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="30" customHeight="1" s="26">
+      <c r="A28" s="12" t="inlineStr">
+        <is>
+          <t>HU-218</t>
+        </is>
+      </c>
+      <c r="B28" s="12" t="inlineStr">
+        <is>
+          <t>EP-21</t>
+        </is>
+      </c>
+      <c r="C28" s="13" t="inlineStr">
+        <is>
+          <t>Atender los tickets de soporte con plazos y encuesta</t>
+        </is>
+      </c>
+      <c r="D28" s="13" t="inlineStr">
+        <is>
+          <t>administrador de SIGMA</t>
+        </is>
+      </c>
+      <c r="E28" s="13" t="inlineStr">
+        <is>
+          <t>gestionar los tickets con prioridad, plazo de respuesta (SLA) y encuesta de satisfacción</t>
+        </is>
+      </c>
+      <c r="F28" s="13" t="inlineStr">
+        <is>
+          <t>cumplir lo prometido al cliente y medir la calidad del servicio</t>
+        </is>
+      </c>
+      <c r="G28" s="12" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="H28" s="12" t="n">
+        <v>80</v>
+      </c>
+      <c r="I28" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="J28" s="12" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="K28" s="13" t="inlineStr">
+        <is>
+          <t>HU-217</t>
+        </is>
+      </c>
+      <c r="L28" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="M28" s="12" t="inlineStr">
+        <is>
+          <t>Terminada</t>
+        </is>
+      </c>
+      <c r="N28" s="13" t="inlineStr">
+        <is>
+          <t>Bryan Chávez</t>
+        </is>
+      </c>
+      <c r="O28" s="12">
+        <f>IF($M28="Terminada",$I28,0)</f>
+        <v/>
+      </c>
+      <c r="P28" s="13" t="inlineStr">
+        <is>
+          <t>Aviso por la campana existente (9 tipos SOPORTE *); job SOPORTE_SLA cada 5 minutos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="30" customHeight="1" s="26">
+      <c r="A29" s="12" t="inlineStr">
+        <is>
+          <t>HU-219</t>
+        </is>
+      </c>
+      <c r="B29" s="12" t="inlineStr">
+        <is>
+          <t>EP-21</t>
+        </is>
+      </c>
+      <c r="C29" s="13" t="inlineStr">
+        <is>
+          <t>Comunicar novedades con campañas segmentadas</t>
+        </is>
+      </c>
+      <c r="D29" s="13" t="inlineStr">
+        <is>
+          <t>administrador de SIGMA</t>
+        </is>
+      </c>
+      <c r="E29" s="13" t="inlineStr">
+        <is>
+          <t>publicar un aviso (banner, modal o tarjeta) a un grupo de usuarios definido por estado, perfil, cliente o planta</t>
+        </is>
+      </c>
+      <c r="F29" s="13" t="inlineStr">
+        <is>
+          <t>informar cambios y novedades solo a quienes les corresponden</t>
+        </is>
+      </c>
+      <c r="G29" s="12" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="H29" s="12" t="n">
+        <v>65</v>
+      </c>
+      <c r="I29" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="J29" s="12" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="K29" s="13" t="inlineStr">
+        <is>
+          <t>HU-217</t>
+        </is>
+      </c>
+      <c r="L29" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="M29" s="12" t="inlineStr">
+        <is>
+          <t>Terminada</t>
+        </is>
+      </c>
+      <c r="N29" s="13" t="inlineStr">
+        <is>
+          <t>Bryan Chávez</t>
+        </is>
+      </c>
+      <c r="O29" s="12">
+        <f>IF($M29="Terminada",$I29,0)</f>
+        <v/>
+      </c>
+      <c r="P29" s="13" t="inlineStr">
+        <is>
+          <t>FNC_CAMPANA_AUDIENCIA admite es/no es y Y/O; entrega por banner, modal, card y la campana. BD/381–383 corregidos por QUOTED_IDENTIFIER.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="30" customHeight="1" s="26">
+      <c r="A30" s="12" t="inlineStr">
+        <is>
+          <t>HU-220</t>
+        </is>
+      </c>
+      <c r="B30" s="12" t="inlineStr">
+        <is>
+          <t>EP-06</t>
+        </is>
+      </c>
+      <c r="C30" s="13" t="inlineStr">
+        <is>
+          <t>Recorrer y operar la bodega en 3D (SIGMA Twin)</t>
+        </is>
+      </c>
+      <c r="D30" s="13" t="inlineStr">
+        <is>
+          <t>bodeguero</t>
+        </is>
+      </c>
+      <c r="E30" s="13" t="inlineStr">
+        <is>
+          <t>ver mis bodegas como un gemelo digital, preparar un picking y contar desde el recorrido</t>
+        </is>
+      </c>
+      <c r="F30" s="13" t="inlineStr">
+        <is>
+          <t>ubicar cada repuesto sin buscar y mantener el inventario exacto</t>
+        </is>
+      </c>
+      <c r="G30" s="12" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="H30" s="12" t="n">
+        <v>85</v>
+      </c>
+      <c r="I30" s="12" t="n">
+        <v>8</v>
+      </c>
+      <c r="J30" s="12" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="K30" s="13" t="inlineStr">
+        <is>
+          <t>HU-050, HU-059</t>
+        </is>
+      </c>
+      <c r="L30" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="M30" s="12" t="inlineStr">
+        <is>
+          <t>Terminada</t>
+        </is>
+      </c>
+      <c r="N30" s="13" t="inlineStr">
+        <is>
+          <t>Bryan Chávez</t>
+        </is>
+      </c>
+      <c r="O30" s="12">
+        <f>IF($M30="Terminada",$I30,0)</f>
+        <v/>
+      </c>
+      <c r="P30" s="13" t="inlineStr">
+        <is>
+          <t>SIGMA Twin: Three.js incluido en Js/three (sin CDN); racks por pasillo con la convención del mapa; picking FEFO/FIFO/LIFO y conteo cíclico (BD/325–336).</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="30" customHeight="1" s="26">
+      <c r="A31" s="12" t="inlineStr">
+        <is>
+          <t>HU-221</t>
+        </is>
+      </c>
+      <c r="B31" s="12" t="inlineStr">
+        <is>
+          <t>EP-18</t>
+        </is>
+      </c>
+      <c r="C31" s="13" t="inlineStr">
+        <is>
+          <t>Ver mi inicio con accesos, alertas y SIGMA AI</t>
+        </is>
+      </c>
+      <c r="D31" s="13" t="inlineStr">
+        <is>
+          <t>usuario de SIGMA</t>
+        </is>
+      </c>
+      <c r="E31" s="13" t="inlineStr">
+        <is>
+          <t>un inicio con mis accesos directos, mis indicadores, mi turno y lo que requiere mi atención</t>
+        </is>
+      </c>
+      <c r="F31" s="13" t="inlineStr">
+        <is>
+          <t>empezar el día sabiendo qué hacer sin recorrer menús</t>
+        </is>
+      </c>
+      <c r="G31" s="12" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="H31" s="12" t="n">
+        <v>80</v>
+      </c>
+      <c r="I31" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="J31" s="12" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="K31" s="13" t="inlineStr">
+        <is>
+          <t>HU-006</t>
+        </is>
+      </c>
+      <c r="L31" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="M31" s="12" t="inlineStr">
+        <is>
+          <t>Terminada</t>
+        </is>
+      </c>
+      <c r="N31" s="13" t="inlineStr">
+        <is>
+          <t>Bryan Chávez</t>
+        </is>
+      </c>
+      <c r="O31" s="12">
+        <f>IF($M31="Terminada",$I31,0)</f>
+        <v/>
+      </c>
+      <c r="P31" s="13" t="inlineStr">
+        <is>
+          <t>Default.aspx con WsInicio (BD/377): accesos por persona, widget SIGMA AI con crear OT en 2 clics, OT recientes, hoy en tu turno y requieren tu atención.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="15" customHeight="1" s="26">
+      <c r="A32" s="15" t="n"/>
+      <c r="B32" s="15" t="n"/>
+      <c r="C32" s="16" t="inlineStr">
         <is>
           <t>Total Sprint 5</t>
         </is>
       </c>
-      <c r="D20" s="16" t="n"/>
-      <c r="E20" s="16" t="n"/>
-      <c r="F20" s="16" t="n"/>
-      <c r="G20" s="15" t="n"/>
-      <c r="H20" s="15" t="n"/>
-      <c r="I20" s="15">
+      <c r="D32" s="16" t="n"/>
+      <c r="E32" s="16" t="n"/>
+      <c r="F32" s="16" t="n"/>
+      <c r="G32" s="15" t="n"/>
+      <c r="H32" s="15" t="n"/>
+      <c r="I32" s="15">
         <f>SUM(I6:I31)</f>
         <v/>
       </c>
-      <c r="J20" s="15" t="n"/>
-      <c r="K20" s="16" t="n"/>
-      <c r="L20" s="15" t="n"/>
-      <c r="M20" s="15" t="n"/>
-      <c r="N20" s="16" t="n"/>
-      <c r="O20" s="15">
+      <c r="J32" s="15" t="n"/>
+      <c r="K32" s="16" t="n"/>
+      <c r="L32" s="15" t="n"/>
+      <c r="M32" s="15" t="n"/>
+      <c r="N32" s="16" t="n"/>
+      <c r="O32" s="15">
         <f>SUM(O6:O31)</f>
         <v/>
       </c>
-      <c r="P20" s="16" t="n"/>
-    </row>
-    <row r="21" ht="30" customHeight="1" s="26"/>
-    <row r="22" ht="30" customHeight="1" s="26"/>
-    <row r="23" ht="30" customHeight="1" s="26"/>
-    <row r="24" ht="30" customHeight="1" s="26"/>
-    <row r="25" ht="30" customHeight="1" s="26"/>
-    <row r="26" ht="30" customHeight="1" s="26"/>
-    <row r="27" ht="30" customHeight="1" s="26"/>
-    <row r="28" ht="30" customHeight="1" s="26"/>
-    <row r="29" ht="30" customHeight="1" s="26"/>
-    <row r="30" ht="30" customHeight="1" s="26"/>
-    <row r="31" ht="30" customHeight="1" s="26"/>
-    <row r="32" ht="15" customHeight="1" s="26"/>
+      <c r="P32" s="16" t="n"/>
+    </row>
   </sheetData>
   <autoFilter ref="A5:P31"/>
   <mergeCells count="2">
@@ -60006,7 +62942,7 @@
       </c>
       <c r="M6" s="9" t="inlineStr">
         <is>
-          <t>Por hacer</t>
+          <t>En revisión</t>
         </is>
       </c>
       <c r="N6" s="10" t="n"/>
@@ -60014,7 +62950,11 @@
         <f>IF($M6="Terminada",$I6,0)</f>
         <v/>
       </c>
-      <c r="P6" s="10" t="n"/>
+      <c r="P6" s="10" t="inlineStr">
+        <is>
+          <t>Avance web al 16-10-2026: Inicio con el widget SIGMA AI (predicciones vigentes con anillo, razones y curva) y el Centro de monitoreo 3D (View/SigmaAI/Centro.aspx, WsAiCentro, BD/379). Falta el panel compacto de la app (CA5).</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="30" customHeight="1" s="26">
       <c r="A7" s="12" t="inlineStr">
@@ -60073,7 +63013,7 @@
       </c>
       <c r="M7" s="12" t="inlineStr">
         <is>
-          <t>Por hacer</t>
+          <t>En revisión</t>
         </is>
       </c>
       <c r="N7" s="13" t="n"/>
@@ -60081,7 +63021,11 @@
         <f>IF($M7="Terminada",$I7,0)</f>
         <v/>
       </c>
-      <c r="P7" s="13" t="n"/>
+      <c r="P7" s="13" t="inlineStr">
+        <is>
+          <t>Avance web al 16-10-2026: Crear OT en 2 clics desde la predicción (WsAlertas.GenerarOrden) con origen predicción y razones precargadas. Falta la fecha propuesta editable (CA2) y el descarte con motivo de 10 caracteres (CA4).</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="30" customHeight="1" s="26">
       <c r="A8" s="9" t="inlineStr">
@@ -60140,7 +63084,7 @@
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>Por hacer</t>
+          <t>En revisión</t>
         </is>
       </c>
       <c r="N8" s="10" t="n"/>
@@ -60148,7 +63092,11 @@
         <f>IF($M8="Terminada",$I8,0)</f>
         <v/>
       </c>
-      <c r="P8" s="10" t="n"/>
+      <c r="P8" s="10" t="inlineStr">
+        <is>
+          <t>Avance web al 16-10-2026: El detalle de la predicción muestra razones ordenadas por peso (SEL_AI_DETALLE) y el Copiloto las explica con reglas. Falta el intervalo de la estimación con su confianza (CA3) y la serie de la variable determinante con banda normal (CA2).</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="30" customHeight="1" s="26">
       <c r="A9" s="12" t="inlineStr">
@@ -60408,7 +63356,7 @@
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>Por hacer</t>
+          <t>En revisión</t>
         </is>
       </c>
       <c r="N12" s="10" t="n"/>
@@ -60416,7 +63364,11 @@
         <f>IF($M12="Terminada",$I12,0)</f>
         <v/>
       </c>
-      <c r="P12" s="10" t="n"/>
+      <c r="P12" s="10" t="inlineStr">
+        <is>
+          <t>Avance web al 16-10-2026: Operación › Cumplimiento (BD/402) mide ocurrencias completadas sobre programadas contra la fecha original, por mes, por plan y por activo (CA1 y CA3). El desglose completo (CA2) tiene completadas y atrasadas; faltan reprogramadas y omitidas por separado.</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="30" customHeight="1" s="26">
       <c r="A13" s="12" t="inlineStr">
@@ -60609,7 +63561,7 @@
       </c>
       <c r="M15" s="12" t="inlineStr">
         <is>
-          <t>Por hacer</t>
+          <t>En revisión</t>
         </is>
       </c>
       <c r="N15" s="13" t="n"/>
@@ -60617,7 +63569,11 @@
         <f>IF($M15="Terminada",$I15,0)</f>
         <v/>
       </c>
-      <c r="P15" s="13" t="n"/>
+      <c r="P15" s="13" t="inlineStr">
+        <is>
+          <t>Avance web al 16-10-2026: Centro de carga de datos (Utilidades › Carga de datos): plantilla con ejemplo, revisión sin escribir y carga confirmada para Inventario, Activos y Mantenimiento (BD/334, 335, 368, 473). Cubre CA1, CA3 y CA4. Falta CA2: avisar que el archivo ya se cargó (hoy volver a cargar no duplica porque los códigos actualizan u omiten).</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="30" customHeight="1" s="26">
       <c r="A16" s="9" t="inlineStr">
@@ -60676,7 +63632,7 @@
       </c>
       <c r="M16" s="9" t="inlineStr">
         <is>
-          <t>Por hacer</t>
+          <t>En revisión</t>
         </is>
       </c>
       <c r="N16" s="10" t="n"/>
@@ -60684,7 +63640,11 @@
         <f>IF($M16="Terminada",$I16,0)</f>
         <v/>
       </c>
-      <c r="P16" s="10" t="n"/>
+      <c r="P16" s="10" t="inlineStr">
+        <is>
+          <t>Avance web al 16-10-2026: La campana y «Requieren tu atención» unen alertas por severidad y antigüedad, y la alerta no crea trabajo sola (CA1 y CA3); se atiende o descarta con motivo. Falta la hoja propia de la bandeja con filtros y exportación.</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="30" customHeight="1" s="26">
       <c r="A17" s="12" t="inlineStr">
@@ -60743,7 +63703,7 @@
       </c>
       <c r="M17" s="12" t="inlineStr">
         <is>
-          <t>Por hacer</t>
+          <t>En revisión</t>
         </is>
       </c>
       <c r="N17" s="13" t="n"/>
@@ -60751,7 +63711,11 @@
         <f>IF($M17="Terminada",$I17,0)</f>
         <v/>
       </c>
-      <c r="P17" s="13" t="n"/>
+      <c r="P17" s="13" t="inlineStr">
+        <is>
+          <t>Avance web al 16-10-2026: Cada celda con error se informa con hoja, fila, columna, valor y motivo, y una fila mala no detiene la carga (CA1 y CA4). Falta corregir la celda dentro de la pantalla y aplicar la corrección a todas las coincidencias (CA2 y CA3): hoy se corrige en la planilla y se revisa de nuevo.</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="30" customHeight="1" s="26">
       <c r="A18" s="9" t="inlineStr">
@@ -60810,7 +63774,7 @@
       </c>
       <c r="M18" s="9" t="inlineStr">
         <is>
-          <t>Por hacer</t>
+          <t>En revisión</t>
         </is>
       </c>
       <c r="N18" s="10" t="n"/>
@@ -60818,7 +63782,11 @@
         <f>IF($M18="Terminada",$I18,0)</f>
         <v/>
       </c>
-      <c r="P18" s="10" t="n"/>
+      <c r="P18" s="10" t="inlineStr">
+        <is>
+          <t>Avance web al 16-10-2026: El módulo Mantenimiento carga frecuencias, tareas, checklists, planes, hitos, actividades y equipos (BD/473) y el plan queda en borrador salvo ACTIVAR = SI (CA1 y CA3). Falta que una frecuencia ambigua pida elegir la interpretación (CA2): hoy se rechaza con el motivo.</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="30" customHeight="1" s="26">
       <c r="A19" s="12" t="inlineStr">
@@ -61279,7 +64247,7 @@
       </c>
       <c r="M25" s="12" t="inlineStr">
         <is>
-          <t>Por hacer</t>
+          <t>En revisión</t>
         </is>
       </c>
       <c r="N25" s="13" t="n"/>
@@ -61287,7 +64255,11 @@
         <f>IF($M25="Terminada",$I25,0)</f>
         <v/>
       </c>
-      <c r="P25" s="13" t="n"/>
+      <c r="P25" s="13" t="inlineStr">
+        <is>
+          <t>Avance web al 16-10-2026: El historial de cargas guarda cada revisión y carga con archivo, fecha, usuario, módulo y resultado, y permite alertar un problema (CA1). El detalle por registro creado (CA2) queda como resumen por hoja.</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="15" customHeight="1" s="26">
       <c r="A26" s="9" t="inlineStr">

</xml_diff>

<commit_message>
Fase 2: web pendiente (indicadores, desempeno de SIGMA AI, carga de datos) reflejada en Sprint 6, informes de prueba, pendientes y bitacora
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Fase 2/Evidencias Proyecto/SIGMA_Product_Backlog_por_Sprint.xlsx
+++ b/Fase 2/Evidencias Proyecto/SIGMA_Product_Backlog_por_Sprint.xlsx
@@ -62952,7 +62952,7 @@
       </c>
       <c r="P6" s="10" t="inlineStr">
         <is>
-          <t>Avance web al 16-10-2026: Inicio con el widget SIGMA AI (predicciones vigentes con anillo, razones y curva) y el Centro de monitoreo 3D (View/SigmaAI/Centro.aspx, WsAiCentro, BD/379). Falta el panel compacto de la app (CA5).</t>
+          <t>Avance web al 17-10-2026: Inicio con el widget SIGMA AI (predicciones vigentes con anillo, razones y curva) y el Centro de monitoreo 3D (View/SigmaAI/Centro.aspx, WsAiCentro, BD/379). Falta el panel compacto de la app (CA5).</t>
         </is>
       </c>
     </row>
@@ -63023,7 +63023,7 @@
       </c>
       <c r="P7" s="13" t="inlineStr">
         <is>
-          <t>Avance web al 16-10-2026: Crear OT en 2 clics desde la predicción (WsAlertas.GenerarOrden) con origen predicción y razones precargadas. Falta la fecha propuesta editable (CA2) y el descarte con motivo de 10 caracteres (CA4).</t>
+          <t>Avance web al 17-10-2026: Crear OT en 2 clics desde la predicción (WsAlertas.GenerarOrden) con origen predicción y razones precargadas. La fecha programada propuesta (CA2) se dejó fuera a propósito: BD/117 decide que programar es una decisión de planificación con dotación y repuestos a la vista. El descarte pide motivo de una lista más detalle opcional, no 10 caracteres (CA4).</t>
         </is>
       </c>
     </row>
@@ -63094,7 +63094,7 @@
       </c>
       <c r="P8" s="10" t="inlineStr">
         <is>
-          <t>Avance web al 16-10-2026: El detalle de la predicción muestra razones ordenadas por peso (SEL_AI_DETALLE) y el Copiloto las explica con reglas. Falta el intervalo de la estimación con su confianza (CA3) y la serie de la variable determinante con banda normal (CA2).</t>
+          <t>Avance web al 17-10-2026: El detalle de la predicción muestra razones ordenadas por peso (SEL_AI_DETALLE) y el Copiloto las explica con reglas. Falta el intervalo de la estimación con su confianza (CA3) y la serie de la variable determinante con banda normal (CA2).</t>
         </is>
       </c>
     </row>
@@ -63155,15 +63155,23 @@
       </c>
       <c r="M9" s="12" t="inlineStr">
         <is>
-          <t>Por hacer</t>
-        </is>
-      </c>
-      <c r="N9" s="13" t="n"/>
+          <t>Terminada</t>
+        </is>
+      </c>
+      <c r="N9" s="13" t="inlineStr">
+        <is>
+          <t>Bryan Chávez</t>
+        </is>
+      </c>
       <c r="O9" s="12">
         <f>IF($M9="Terminada",$I9,0)</f>
         <v/>
       </c>
-      <c r="P9" s="13" t="n"/>
+      <c r="P9" s="13" t="inlineStr">
+        <is>
+          <t>Avance web al 17-10-2026: Mantenimiento › Indicadores › Tablero (BD/474, WsIndicadores): cumplimiento, disponibilidad, tiempo medio entre fallas, tiempo medio de reparación y órdenes pendientes de cierre con su variación contra el período anterior (CA1); filtros de planta, área, equipo y fechas que recalculan todo (CA2); cada indicador abre su detalle en un cajón (CA3).</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="30" customHeight="1" s="26">
       <c r="A10" s="9" t="inlineStr">
@@ -63289,15 +63297,23 @@
       </c>
       <c r="M11" s="12" t="inlineStr">
         <is>
-          <t>Por hacer</t>
-        </is>
-      </c>
-      <c r="N11" s="13" t="n"/>
+          <t>Terminada</t>
+        </is>
+      </c>
+      <c r="N11" s="13" t="inlineStr">
+        <is>
+          <t>Bryan Chávez</t>
+        </is>
+      </c>
       <c r="O11" s="12">
         <f>IF($M11="Terminada",$I11,0)</f>
         <v/>
       </c>
-      <c r="P11" s="13" t="n"/>
+      <c r="P11" s="13" t="inlineStr">
+        <is>
+          <t>Avance web al 17-10-2026: Pantalla SIGMA AI › Desempeño › «Por evaluar» (View/SigmaAI/Desempeno.aspx, WsAiDesempeno, BD/475): lista las predicciones con el horizonte vencido sin evaluar (CA3), registra si el evento ocurrió y cuándo con el error en días calculado por el SP (CA1) y clasifica «acierto con intervención» aparte de la falsa alarma (CA2).</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="30" customHeight="1" s="26">
       <c r="A12" s="9" t="inlineStr">
@@ -63366,7 +63382,7 @@
       </c>
       <c r="P12" s="10" t="inlineStr">
         <is>
-          <t>Avance web al 16-10-2026: Operación › Cumplimiento (BD/402) mide ocurrencias completadas sobre programadas contra la fecha original, por mes, por plan y por activo (CA1 y CA3). El desglose completo (CA2) tiene completadas y atrasadas; faltan reprogramadas y omitidas por separado.</t>
+          <t>Avance web al 17-10-2026: El tablero y Operación › Cumplimiento miden hechas sobre vencidas contra la fecha original (CA1) y ordenan los equipos del peor al mejor (CA3). El desglose completo (CA2) distingue hechas y vencidas; faltan reprogramadas y omitidas por separado.</t>
         </is>
       </c>
     </row>
@@ -63427,15 +63443,23 @@
       </c>
       <c r="M13" s="12" t="inlineStr">
         <is>
-          <t>Por hacer</t>
-        </is>
-      </c>
-      <c r="N13" s="13" t="n"/>
+          <t>Terminada</t>
+        </is>
+      </c>
+      <c r="N13" s="13" t="inlineStr">
+        <is>
+          <t>Bryan Chávez</t>
+        </is>
+      </c>
       <c r="O13" s="12">
         <f>IF($M13="Terminada",$I13,0)</f>
         <v/>
       </c>
-      <c r="P13" s="13" t="n"/>
+      <c r="P13" s="13" t="inlineStr">
+        <is>
+          <t>Avance web al 17-10-2026: Tablero e indicadores (BD/474): disponibilidad con la indisponibilidad no planificada descontada y la planificada aparte (CA1); tiempo medio entre fallas con aviso cuando hay menos de 3 fallas (CA2); tiempo medio de reparación sobre las correctivas cerradas (CA3).</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="30" customHeight="1" s="26">
       <c r="A14" s="9" t="inlineStr">
@@ -63494,15 +63518,23 @@
       </c>
       <c r="M14" s="9" t="inlineStr">
         <is>
-          <t>Por hacer</t>
-        </is>
-      </c>
-      <c r="N14" s="10" t="n"/>
+          <t>Terminada</t>
+        </is>
+      </c>
+      <c r="N14" s="10" t="inlineStr">
+        <is>
+          <t>Bryan Chávez</t>
+        </is>
+      </c>
       <c r="O14" s="9">
         <f>IF($M14="Terminada",$I14,0)</f>
         <v/>
       </c>
-      <c r="P14" s="10" t="n"/>
+      <c r="P14" s="10" t="inlineStr">
+        <is>
+          <t>Avance web al 17-10-2026: Mantenimiento › Indicadores › Costos (BD/474): repuestos, mano de obra y servicios por equipo y siempre por moneda (CA1); por centro de costo con el de sus dependientes (CA2, probado con un árbol de prueba revertido); comparación con el período anterior en variación absoluta y porcentual (CA3).</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="30" customHeight="1" s="26">
       <c r="A15" s="12" t="inlineStr">
@@ -63561,17 +63593,21 @@
       </c>
       <c r="M15" s="12" t="inlineStr">
         <is>
-          <t>En revisión</t>
-        </is>
-      </c>
-      <c r="N15" s="13" t="n"/>
+          <t>Terminada</t>
+        </is>
+      </c>
+      <c r="N15" s="13" t="inlineStr">
+        <is>
+          <t>Bryan Chávez</t>
+        </is>
+      </c>
       <c r="O15" s="12">
         <f>IF($M15="Terminada",$I15,0)</f>
         <v/>
       </c>
       <c r="P15" s="13" t="inlineStr">
         <is>
-          <t>Avance web al 16-10-2026: Centro de carga de datos (Utilidades › Carga de datos): plantilla con ejemplo, revisión sin escribir y carga confirmada para Inventario, Activos y Mantenimiento (BD/334, 335, 368, 473). Cubre CA1, CA3 y CA4. Falta CA2: avisar que el archivo ya se cargó (hoy volver a cargar no duplica porque los códigos actualizan u omiten).</t>
+          <t>Avance web al 17-10-2026: Centro de carga de datos (BD/334, 335, 368, 473, 476): revisión sin escribir (CA1), aviso de que la planilla ya se procesó, con fecha y usuario, gracias a la huella SHA-256 del archivo (CA2), carga confirmada (CA3) y plantilla con ejemplo (CA4).</t>
         </is>
       </c>
     </row>
@@ -63642,7 +63678,7 @@
       </c>
       <c r="P16" s="10" t="inlineStr">
         <is>
-          <t>Avance web al 16-10-2026: La campana y «Requieren tu atención» unen alertas por severidad y antigüedad, y la alerta no crea trabajo sola (CA1 y CA3); se atiende o descarta con motivo. Falta la hoja propia de la bandeja con filtros y exportación.</t>
+          <t>Avance web al 17-10-2026: La campana y «Requieren tu atención» unen alertas por severidad y antigüedad, y la alerta no crea trabajo sola (CA1 y CA3); se atiende o descarta con motivo. Falta la hoja propia de la bandeja con filtros y exportación.</t>
         </is>
       </c>
     </row>
@@ -63713,7 +63749,7 @@
       </c>
       <c r="P17" s="13" t="inlineStr">
         <is>
-          <t>Avance web al 16-10-2026: Cada celda con error se informa con hoja, fila, columna, valor y motivo, y una fila mala no detiene la carga (CA1 y CA4). Falta corregir la celda dentro de la pantalla y aplicar la corrección a todas las coincidencias (CA2 y CA3): hoy se corrige en la planilla y se revisa de nuevo.</t>
+          <t>Avance web al 17-10-2026: Cada celda con error se informa con hoja, fila, columna, valor y motivo, y una fila mala no detiene la carga (CA1 y CA4). Falta corregir la celda dentro de la pantalla y aplicar la corrección a todas las coincidencias (CA2 y CA3): hoy se corrige en la planilla y se revisa de nuevo.</t>
         </is>
       </c>
     </row>
@@ -63784,7 +63820,7 @@
       </c>
       <c r="P18" s="10" t="inlineStr">
         <is>
-          <t>Avance web al 16-10-2026: El módulo Mantenimiento carga frecuencias, tareas, checklists, planes, hitos, actividades y equipos (BD/473) y el plan queda en borrador salvo ACTIVAR = SI (CA1 y CA3). Falta que una frecuencia ambigua pida elegir la interpretación (CA2): hoy se rechaza con el motivo.</t>
+          <t>Avance web al 17-10-2026: El módulo Mantenimiento carga frecuencias, tareas, checklists, planes, hitos, actividades y equipos (BD/473) y el plan queda en borrador salvo ACTIVAR = SI (CA1 y CA3). Falta que una frecuencia ambigua pida elegir la interpretación (CA2): hoy se rechaza con el motivo.</t>
         </is>
       </c>
     </row>
@@ -64046,7 +64082,7 @@
       </c>
       <c r="M22" s="9" t="inlineStr">
         <is>
-          <t>Por hacer</t>
+          <t>En revisión</t>
         </is>
       </c>
       <c r="N22" s="10" t="n"/>
@@ -64054,7 +64090,11 @@
         <f>IF($M22="Terminada",$I22,0)</f>
         <v/>
       </c>
-      <c r="P22" s="10" t="n"/>
+      <c r="P22" s="10" t="inlineStr">
+        <is>
+          <t>Avance web al 17-10-2026: Excel con los mismos filtros de la pantalla y encabezado de cliente, período y filtros (CA1) e impresión con el pie del cliente (CA2), para el tablero, el detalle de cada indicador y los costos. Falta ofrecerlos en los demás listados de SIGMA (Operación, órdenes, activos).</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="30" customHeight="1" s="26">
       <c r="A23" s="12" t="inlineStr">
@@ -64113,7 +64153,7 @@
       </c>
       <c r="M23" s="12" t="inlineStr">
         <is>
-          <t>Por hacer</t>
+          <t>En revisión</t>
         </is>
       </c>
       <c r="N23" s="13" t="n"/>
@@ -64121,7 +64161,11 @@
         <f>IF($M23="Terminada",$I23,0)</f>
         <v/>
       </c>
-      <c r="P23" s="13" t="n"/>
+      <c r="P23" s="13" t="inlineStr">
+        <is>
+          <t>Avance web al 17-10-2026: Centro de SIGMA AI › Fotos de terreno: cada detección se presenta «por confirmar» y no como confirmada hasta que una persona la confirma o corrige (CA3 y CA4), y esa decisión alimenta el dataset. Falta la cola de análisis con prioridad (CA1) y dibujar las zonas detectadas sobre la imagen (CA2).</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="30" customHeight="1" s="26">
       <c r="A24" s="9" t="inlineStr">
@@ -64180,7 +64224,7 @@
       </c>
       <c r="M24" s="9" t="inlineStr">
         <is>
-          <t>Por hacer</t>
+          <t>En revisión</t>
         </is>
       </c>
       <c r="N24" s="10" t="n"/>
@@ -64188,7 +64232,11 @@
         <f>IF($M24="Terminada",$I24,0)</f>
         <v/>
       </c>
-      <c r="P24" s="10" t="n"/>
+      <c r="P24" s="10" t="inlineStr">
+        <is>
+          <t>Avance web al 17-10-2026: Pestaña «Desempeño» (BD/475): por versión y mes, predicciones, evaluadas, aciertos, falsas alarmas y aciertos con intervención aparte (CA1); la versión queda «candidata a reentrenamiento» si la precisión cae bajo la de referencia con al menos 5 evaluadas (CA2). Falta la desviación de los datos de entrada (CA3): no se guarda la distribución del entrenamiento.</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="30" customHeight="1" s="26">
       <c r="A25" s="12" t="inlineStr">
@@ -64247,17 +64295,21 @@
       </c>
       <c r="M25" s="12" t="inlineStr">
         <is>
-          <t>En revisión</t>
-        </is>
-      </c>
-      <c r="N25" s="13" t="n"/>
+          <t>Terminada</t>
+        </is>
+      </c>
+      <c r="N25" s="13" t="inlineStr">
+        <is>
+          <t>Bryan Chávez</t>
+        </is>
+      </c>
       <c r="O25" s="12">
         <f>IF($M25="Terminada",$I25,0)</f>
         <v/>
       </c>
       <c r="P25" s="13" t="inlineStr">
         <is>
-          <t>Avance web al 16-10-2026: El historial de cargas guarda cada revisión y carga con archivo, fecha, usuario, módulo y resultado, y permite alertar un problema (CA1). El detalle por registro creado (CA2) queda como resumen por hoja.</t>
+          <t>Avance web al 17-10-2026: El historial guarda cada revisión y carga con archivo, fecha, usuario, módulo y resultado (CA1); al abrir una carga se ve el resultado por hoja, con filas, creadas, actualizadas, omitidas y errores (CA2).</t>
         </is>
       </c>
     </row>

</xml_diff>